<commit_message>
Actualizacion de historias de usuario respecto a la planilla de control de cambios
</commit_message>
<xml_diff>
--- a/Fase 2/Evidencias proyecto/Documentación/SCRUM/3. Historias Usuario con instructivo.xlsx
+++ b/Fase 2/Evidencias proyecto/Documentación/SCRUM/3. Historias Usuario con instructivo.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="275" uniqueCount="275">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="284" uniqueCount="284">
   <si>
     <t xml:space="preserve">Desarrollo ágil: Historias de usuario y criterios de aceptación</t>
   </si>
@@ -179,7 +179,7 @@
     <t xml:space="preserve">En caso de que el dataset presente registros incompletos o mediciones fuera de rango biológico</t>
   </si>
   <si>
-    <t xml:space="preserve">cuando se ejecuta el script de limpieza sobre los datos crudos</t>
+    <t xml:space="preserve">cuando se ejecuta el script de limpieza sobre el dataset crudo</t>
   </si>
   <si>
     <t xml:space="preserve">las celdas nulas quedan imputadas según la regla definida y los registros anómalos son filtrados sin dejar vacíos residuales.</t>
@@ -212,6 +212,132 @@
     <t>HU-05</t>
   </si>
   <si>
+    <t xml:space="preserve">Como cientifico de datos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">necesito tener un dataset completo y enriquecido, más allá de las mediciones </t>
+  </si>
+  <si>
+    <t xml:space="preserve">para trabajar con un elemento eficiente.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Integracion de los 3 datasets</t>
+  </si>
+  <si>
+    <t xml:space="preserve">En caso de requerir mayor informacion </t>
+  </si>
+  <si>
+    <t xml:space="preserve">cuando se complemente el dataset de frutos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">se genera un dataset completo, resultado de la unión de 3 datasets distintos.</t>
+  </si>
+  <si>
+    <t>HU-06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">necesitamos estructurar el Documento de Arquitectura de Software (DAS) con diagramas de alto y bajo nivel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Con la finalidad de definir la interacción técnica entre la interfaz web, el backend, la API de inferencia y el modelo serializado previo a su construcción.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Modelado de arquitectura de alto nivel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">En caso de requerir representar la vista global del sistema y sus límites</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cuando se elaboran los diagramas de contexto </t>
+  </si>
+  <si>
+    <t xml:space="preserve">quedan formalmente identificadas las comunicaciones entre el usuario web, el servidor de aplicaciones y los archivos del modelo en el DAS.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Diseño de componentes y flujo de inferencia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">En caso de definir el funcionamiento interno de la API y el preprocesamiento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cuando se grafican los diagramas de componentes o secuencia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">se documenta con precisión la ruta de los datos desde la petición HTTP, el vector de entrada, la llamada al pipeline serializado y el formato de respuesta JSON.</t>
+  </si>
+  <si>
+    <t>HU-07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como docente evaluador </t>
+  </si>
+  <si>
+    <t xml:space="preserve">necesito disponer de una interfaz visual que represente el funcionamiento del modelo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">para tener certeza de como va a ser el modelo y su funcionamiento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Diseño de interfaz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">En caso de representar los campos de entrada y salida del modelo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cuando se diseña el formulario de entrada y el contenedor de la salida de la simulacion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">se dispone de un diseño atractivo, orientado a la usabilidad.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Simulación funcional</t>
+  </si>
+  <si>
+    <t xml:space="preserve">En caso de arrojar una simulación de predicción</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cuando el usuario de prueba le da al boton de predecir</t>
+  </si>
+  <si>
+    <t xml:space="preserve">se visualiza la prediccion del modelo</t>
+  </si>
+  <si>
+    <t>HU-08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">necesito revisar el informe de avance intermedio y los artefactos parciales de datos y experimentación</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Con la finalidad de certificar la continuidad operativa, el ritmo de los Sprints y la viabilidad técnica antes del cierre de la Fase 2.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Revisión de entregables parciales</t>
+  </si>
+  <si>
+    <t xml:space="preserve">En caso de presentar la documentación y notebooks de la primera mitad de la Fase 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cuando la comisión académica evalúa el dataset consolidado y los resultados preliminares del modelamiento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">se valida el cumplimiento de las evidencias de avance comprometidas en el plan de trabajo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Auditoría del flujo ágil</t>
+  </si>
+  <si>
+    <t xml:space="preserve">En caso de auditar la trazabilidad del equipo en Taiga y Github</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cuando se contrastan los gráficos de avance con los compromisos de los Sprints ejecutados</t>
+  </si>
+  <si>
+    <t xml:space="preserve">se aprueba la calificación de avance técnico sin observaciones críticas de bloqueo metodológico.</t>
+  </si>
+  <si>
+    <t>HU-09</t>
+  </si>
+  <si>
     <t xml:space="preserve">necesitamos entrenar de forma comparativa diversos algoritmos de aprendizaje automático con el conjunto de datos limpio</t>
   </si>
   <si>
@@ -239,7 +365,7 @@
     <t xml:space="preserve">cuando se lanza la rutina de ajuste con parámetros base</t>
   </si>
   <si>
-    <t xml:space="preserve">se generan los modelos ajustados sin errores de convergencia ni fallos de memoria en el entorno de ejecución.</t>
+    <t xml:space="preserve">se generan los modelos ajustados con errores de convergencia menores.</t>
   </si>
   <si>
     <t xml:space="preserve">Búsqueda y ajuste de hiperparámetros</t>
@@ -254,7 +380,7 @@
     <t xml:space="preserve">se obtienen las combinaciones óptimas que maximizan el rendimiento.</t>
   </si>
   <si>
-    <t>HU-06</t>
+    <t>HU-10</t>
   </si>
   <si>
     <t xml:space="preserve">necesitamos calcular y comparar las métricas de rendimiento sobre el conjunto de prueba independiente</t>
@@ -287,7 +413,7 @@
     <t xml:space="preserve">queda formalmente documentado y justificado cuál es el algoritmo con mayor rendimiento para la estimación de carga frutal.</t>
   </si>
   <si>
-    <t>HU-07</t>
+    <t>HU-11</t>
   </si>
   <si>
     <t xml:space="preserve">necesitamos empaquetar y serializar el modelo seleccionado junto a sus transformaciones de preprocesamiento en un archivo persistente</t>
@@ -320,7 +446,7 @@
     <t xml:space="preserve">el artefacto cargado procesa las entradas y retorna una predicción numérica válida sin errores de compatibilidad ni dependencias faltantes.</t>
   </si>
   <si>
-    <t>HU-08</t>
+    <t>HU-12</t>
   </si>
   <si>
     <t xml:space="preserve">Como usuario</t>
@@ -368,7 +494,7 @@
     <t xml:space="preserve">la pantalla despliega un formulario ordenado con etiquetas explícitas, indicadores y jerarquía visual clara.</t>
   </si>
   <si>
-    <t>HU-09</t>
+    <t>HU-13</t>
   </si>
   <si>
     <t xml:space="preserve">necesitamos implementar el backend y los endpoints de conexión que reciban los datos del formulario, carguen el modelo serializado y devuelvan la predicción</t>
@@ -401,40 +527,7 @@
     <t xml:space="preserve">el backend retorna una respuesta estructurada con el valor estimado de carga frutal en un tiempo menor a 2 segundos.</t>
   </si>
   <si>
-    <t>HU-10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">necesitamos empaquetar y orquestar los servicios de frontend y backend mediante contenedores Docker</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Con la finalidad de garantizar un despliegue reproducible, aislado y libre de conflictos de dependencias para su evaluación y puesta en marcha.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Orquestación mediante Docker Compose</t>
-  </si>
-  <si>
-    <t xml:space="preserve">En caso de inicializar la plataforma en el equipo anfitrión</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cuando se ejecuta el comando necesario</t>
-  </si>
-  <si>
-    <t xml:space="preserve">el sistema descarga las imágenes base, compila el frontend en Nginx, levanta la API de FastAPI y vincula ambos servicios en una red interna.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Disponibilidad y acceso por puerto publicado</t>
-  </si>
-  <si>
-    <t xml:space="preserve">En caso de que los contenedores se encuentren en ejecución</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cuando un evaluador ingresa desde su navegador a la dirección local asignada</t>
-  </si>
-  <si>
-    <t xml:space="preserve">la interfaz web carga en su totalidad, se comunica transparentemente con el backend y permite realizar consultas de manera estable.</t>
-  </si>
-  <si>
-    <t>HU-11</t>
+    <t>HU-14</t>
   </si>
   <si>
     <t xml:space="preserve">necesitamos realizar pruebas de integración extremo a extremo sobre el flujo completo de consulta web</t>
@@ -467,112 +560,13 @@
     <t xml:space="preserve">la interfaz web despliega un mensaje amigable al usuario evitando caídas de la aplicación o pantallas en blanco.</t>
   </si>
   <si>
-    <t>HU-12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">necesitamos estructurar el Documento de Arquitectura de Software (DAS) con diagramas de alto y bajo nivel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Con la finalidad de definir la interacción técnica entre la interfaz web, el backend, la API de inferencia y el modelo serializado previo a su construcción.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Modelado de arquitectura de alto nivel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">En caso de requerir representar la vista global del sistema y sus límites</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cuando se elaboran los diagramas de contexto </t>
-  </si>
-  <si>
-    <t xml:space="preserve">quedan formalmente identificadas las comunicaciones entre el usuario web, el servidor de aplicaciones y los archivos del modelo en el DAS.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Diseño de componentes y flujo de inferencia</t>
-  </si>
-  <si>
-    <t xml:space="preserve">En caso de definir el funcionamiento interno de la API y el preprocesamiento</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cuando se grafican los diagramas de componentes o secuencia</t>
-  </si>
-  <si>
-    <t xml:space="preserve">se documenta con precisión la ruta de los datos desde la petición HTTP, el vector de entrada, la llamada al pipeline serializado y el formato de respuesta JSON.</t>
-  </si>
-  <si>
-    <t>HU-13</t>
-  </si>
-  <si>
-    <t xml:space="preserve">necesito revisar el informe de avance intermedio y los artefactos parciales de datos y experimentación</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Con la finalidad de certificar la continuidad operativa, el ritmo de los Sprints y la viabilidad técnica antes del cierre de la Fase 2.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Revisión de entregables parciales</t>
-  </si>
-  <si>
-    <t xml:space="preserve">En caso de presentar la documentación y notebooks de la primera mitad de la Fase 2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cuando la comisión académica evalúa el dataset consolidado y los resultados preliminares del modelamiento</t>
-  </si>
-  <si>
-    <t xml:space="preserve">se valida el cumplimiento de las evidencias de avance comprometidas en el plan de trabajo.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Auditoría del flujo ágil</t>
-  </si>
-  <si>
-    <t xml:space="preserve">En caso de auditar la trazabilidad del equipo en Taiga y Codeberg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cuando se contrastan los gráficos de avance con los compromisos de los Sprints ejecutados</t>
-  </si>
-  <si>
-    <t xml:space="preserve">se aprueba la calificación de avance técnico sin observaciones críticas de bloqueo metodológico.</t>
-  </si>
-  <si>
-    <t>HU-14</t>
-  </si>
-  <si>
-    <t xml:space="preserve">necesito examinar la solución integral terminada, el informe final consolidado y el código fuente documentado</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Con la finalidad de calificar el cumplimiento de las competencias del perfil de egreso y dar por aprobada la Fase 2 del proyecto de titulación.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Evaluación de entregables de cierre</t>
-  </si>
-  <si>
-    <t xml:space="preserve">En caso de concluir el Sprint 3 con la plataforma web desplegada y el modelo integrado</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cuando la comisión revisa el informe técnico final y la ejecución del sistema en vivo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">se certifica el funcionamiento del producto de software conforme a los objetivos general y específicos planteados.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Inspección de repositorios y calidad de ingeniería</t>
-  </si>
-  <si>
-    <t xml:space="preserve">En caso de auditar la entrega final del proyecto</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cuando se examina la estructura del repositorio en Codeberg y las pruebas de validación</t>
-  </si>
-  <si>
-    <t xml:space="preserve">queda acreditada la calidad del código, el desacoplamiento de componentes y la documentación metodológica completa.</t>
-  </si>
-  <si>
     <t>HU-15</t>
   </si>
   <si>
     <t xml:space="preserve">Como usuario interesado </t>
   </si>
   <si>
-    <t xml:space="preserve">necesito registrar una cuenta mediante correo electrónico y contraseña en el formulario web.</t>
+    <t xml:space="preserve">necesito registrar una cuenta mediante correo electrónico y contraseña, e iniciar sesión con mis credenciales y poder cerrar mi sesión cuando lo decida.</t>
   </si>
   <si>
     <t xml:space="preserve">Con la finalidad de disponer de credenciales personales para acceder a las funciones del sistema.</t>
@@ -590,18 +584,6 @@
     <t xml:space="preserve">el sistema crea la cuenta en el servicio de autenticación, notifica el éxito del proceso y redirige a la vista de inicio de sesión.</t>
   </si>
   <si>
-    <t xml:space="preserve">Intento de registro con correo duplicado</t>
-  </si>
-  <si>
-    <t xml:space="preserve">En caso de que se intente crear una cuenta utilizando una dirección de correo electrónico que ya se encuentra registrada en el sistema</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cuando se envía la solicitud de registro</t>
-  </si>
-  <si>
-    <t xml:space="preserve">el sistema rechaza la creación de la cuenta y muestra un mensaje de alerta indicando que el correo ya está en uso.</t>
-  </si>
-  <si>
     <t xml:space="preserve">Validación de formato de credenciales</t>
   </si>
   <si>
@@ -612,18 +594,6 @@
   </si>
   <si>
     <t xml:space="preserve">el sistema bloquea el envío de la petición y resalta los campos con error indicando las reglas que deben cumplirse.</t>
-  </si>
-  <si>
-    <t>HU-16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Como usuario registrado.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">necesito iniciar sesión con mis credenciales y poder cerrar mi sesión cuando lo decida.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Con la finalidad de acceder a la plataforma de forma identificada y resguardar mi sesión activa.</t>
   </si>
   <si>
     <t xml:space="preserve">Inicio de sesión correcto</t>
@@ -662,7 +632,7 @@
     <t xml:space="preserve">el sistema destruye el token o estado de sesión local y redirige la vista a la pantalla principal o de acceso público.</t>
   </si>
   <si>
-    <t>HU-17</t>
+    <t>HU-16</t>
   </si>
   <si>
     <t xml:space="preserve">Como sistema</t>
@@ -710,7 +680,7 @@
     <t xml:space="preserve">el sistema rechaza la petición con un código de no autorización y solicita reiniciar la sesión.</t>
   </si>
   <si>
-    <t>HU-18</t>
+    <t>HU-17</t>
   </si>
   <si>
     <t xml:space="preserve">Como administrador del sistema</t>
@@ -758,7 +728,7 @@
     <t xml:space="preserve">el sistema lista las consultas efectuadas a nivel global indicando fecha, identificador o correo del usuario, variables de entrada y el resultado estimado calculado.</t>
   </si>
   <si>
-    <t>HU-19</t>
+    <t>HU-18</t>
   </si>
   <si>
     <t xml:space="preserve">Como usuario autenticado</t>
@@ -804,6 +774,63 @@
   </si>
   <si>
     <t xml:space="preserve">el sistema presenta los datos de forma paginada o estructurada en un tiempo inferior a 2 segundos bajo condiciones nominales.</t>
+  </si>
+  <si>
+    <t>HU-19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">necesito examinar la solución integral terminada, el informe final consolidado y el código fuente documentado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Con la finalidad de calificar el cumplimiento de las competencias del perfil de egreso y dar por aprobada la Fase 2 del proyecto de titulación.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Evaluación de entregables de cierre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">En caso de concluir el Sprint 3 con la plataforma web desplegada y el modelo integrado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cuando la comisión revisa el informe técnico final y la ejecución del sistema en vivo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">se certifica el funcionamiento del producto de software conforme a los objetivos general y específicos planteados.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inspección de repositorios y calidad de ingeniería</t>
+  </si>
+  <si>
+    <t xml:space="preserve">En caso de auditar la entrega final del proyecto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cuando se examina la estructura del repositorio en Codeberg y las pruebas de validación</t>
+  </si>
+  <si>
+    <t xml:space="preserve">queda acreditada la calidad del código, el desacoplamiento de componentes y la documentación metodológica completa.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Orquestación mediante Docker Compose</t>
+  </si>
+  <si>
+    <t xml:space="preserve">En caso de inicializar la plataforma en el equipo anfitrión</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cuando se ejecuta el comando necesario</t>
+  </si>
+  <si>
+    <t xml:space="preserve">el sistema descarga las imágenes base, compila el frontend en Nginx, levanta la API de FastAPI y vincula ambos servicios en una red interna.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Disponibilidad y acceso por puerto publicado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">En caso de que los contenedores se encuentren en ejecución</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cuando un evaluador ingresa desde su navegador a la dirección local asignada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">la interfaz web carga en su totalidad, se comunica transparentemente con el backend y permite realizar consultas de manera estable.</t>
   </si>
   <si>
     <t xml:space="preserve">Historias de usuario y criterios de aceptación: Instructivo</t>
@@ -856,7 +883,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <sz val="11.000000"/>
       <color theme="1"/>
@@ -892,13 +919,16 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11.000000"/>
+    </font>
+    <font>
       <b/>
       <sz val="24.000000"/>
       <color theme="1"/>
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="13">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -919,8 +949,20 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="2" tint="-0.049989318521683403"/>
+        <bgColor theme="2" tint="-0.049989318521683403"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFD8D8D8"/>
         <bgColor rgb="FFD8D8D8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.59999389629810485"/>
+        <bgColor theme="4" tint="0.59999389629810485"/>
       </patternFill>
     </fill>
     <fill>
@@ -929,8 +971,38 @@
         <bgColor rgb="FFB7B7B7"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.59999389629810485"/>
+        <bgColor theme="6" tint="0.59999389629810485"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor theme="7" tint="0.79998168889431442"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-0.14999847407452621"/>
+        <bgColor theme="2" tint="-0.14999847407452621"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="0"/>
+        <bgColor theme="0" tint="0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-0.249977111117893"/>
+        <bgColor theme="2" tint="-0.249977111117893"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="8">
+  <borders count="11">
     <border>
       <left style="none"/>
       <right style="none"/>
@@ -1027,11 +1099,48 @@
       <bottom style="none"/>
       <diagonal style="none"/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="76">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment readingOrder="0"/>
     </xf>
@@ -1059,7 +1168,7 @@
     <xf fontId="4" fillId="3" borderId="4" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf fontId="1" fillId="2" borderId="5" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="1" fillId="4" borderId="5" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" readingOrder="0" vertical="center" wrapText="1"/>
     </xf>
     <xf fontId="1" fillId="2" borderId="5" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1071,6 +1180,7 @@
     <xf fontId="1" fillId="2" borderId="4" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" readingOrder="0" vertical="center" wrapText="1"/>
     </xf>
+    <xf fontId="5" fillId="4" borderId="6" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf fontId="5" fillId="0" borderId="6" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf fontId="1" fillId="2" borderId="4" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" readingOrder="0" vertical="center" wrapText="1"/>
@@ -1078,32 +1188,88 @@
     <xf fontId="1" fillId="4" borderId="7" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf fontId="1" fillId="4" borderId="7" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="1" fillId="5" borderId="7" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf fontId="1" fillId="4" borderId="4" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="1" fillId="5" borderId="4" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf fontId="1" fillId="4" borderId="4" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="1" fillId="5" borderId="4" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf fontId="6" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment readingOrder="0" vertical="center" wrapText="1"/>
     </xf>
+    <xf fontId="1" fillId="5" borderId="7" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="1" fillId="6" borderId="5" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="5" fillId="6" borderId="6" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf fontId="1" fillId="6" borderId="4" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="5" fillId="6" borderId="7" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf fontId="5" fillId="0" borderId="7" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf fontId="1" fillId="5" borderId="4" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="1" fillId="2" borderId="5" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="1" fillId="6" borderId="4" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf fontId="1" fillId="5" borderId="4" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="1" fillId="7" borderId="4" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf fontId="1" fillId="5" borderId="4" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="1" fillId="7" borderId="4" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="1" fillId="6" borderId="5" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="1" fillId="2" borderId="8" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="1" fillId="2" borderId="4" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="5" fillId="6" borderId="9" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf fontId="5" fillId="6" borderId="9" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="7" fillId="0" borderId="9" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="1" fillId="6" borderId="5" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf fontId="1" fillId="7" borderId="5" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf fontId="1" fillId="2" borderId="9" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="1" fillId="7" borderId="5" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf fontId="1" fillId="7" borderId="5" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="1" fillId="8" borderId="5" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf fontId="1" fillId="2" borderId="5" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf fontId="1" fillId="8" borderId="7" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf fontId="1" fillId="2" borderId="7" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="1" fillId="8" borderId="6" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf fontId="1" fillId="2" borderId="6" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1112,19 +1278,55 @@
     <xf fontId="6" fillId="0" borderId="4" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment readingOrder="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf fontId="1" fillId="0" borderId="5" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="1" fillId="8" borderId="4" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf fontId="1" fillId="8" borderId="5" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" readingOrder="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf fontId="1" fillId="0" borderId="5" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="5" fillId="8" borderId="6" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf fontId="1" fillId="7" borderId="4" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf fontId="1" fillId="9" borderId="5" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="5" fillId="9" borderId="7" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf fontId="5" fillId="9" borderId="6" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf fontId="1" fillId="9" borderId="4" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf fontId="1" fillId="9" borderId="8" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="1" fillId="9" borderId="9" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="1" fillId="9" borderId="10" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="1" fillId="2" borderId="10" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="5" fillId="10" borderId="7" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf fontId="1" fillId="10" borderId="4" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="1" fillId="10" borderId="4" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="11" borderId="0" numFmtId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf fontId="1" fillId="11" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf fontId="5" fillId="12" borderId="7" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf fontId="1" fillId="12" borderId="4" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="1" fillId="12" borderId="4" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" readingOrder="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf fontId="1" fillId="0" borderId="4" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="1" fillId="0" borderId="4" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" readingOrder="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="7" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf fontId="8" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf fontId="3" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf fontId="4" fillId="3" borderId="4" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf fontId="1" fillId="2" borderId="4" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1859,10 +2061,10 @@
     <row r="7" ht="28.5">
       <c r="A7" s="1"/>
       <c r="B7" s="15"/>
-      <c r="C7" s="15"/>
-      <c r="D7" s="15"/>
-      <c r="E7" s="15"/>
-      <c r="F7" s="16">
+      <c r="C7" s="16"/>
+      <c r="D7" s="16"/>
+      <c r="E7" s="16"/>
+      <c r="F7" s="17">
         <v>2</v>
       </c>
       <c r="G7" s="14" t="s">
@@ -1896,15 +2098,15 @@
     </row>
     <row r="8" ht="14.25" customHeight="1">
       <c r="A8" s="1"/>
-      <c r="B8" s="17"/>
-      <c r="C8" s="18"/>
-      <c r="D8" s="18"/>
-      <c r="E8" s="18"/>
-      <c r="F8" s="19"/>
-      <c r="G8" s="20"/>
-      <c r="H8" s="20"/>
-      <c r="I8" s="20"/>
-      <c r="J8" s="20"/>
+      <c r="B8" s="18"/>
+      <c r="C8" s="19"/>
+      <c r="D8" s="19"/>
+      <c r="E8" s="19"/>
+      <c r="F8" s="20"/>
+      <c r="G8" s="21"/>
+      <c r="H8" s="21"/>
+      <c r="I8" s="21"/>
+      <c r="J8" s="21"/>
       <c r="K8" s="1"/>
       <c r="L8" s="1"/>
       <c r="M8" s="1"/>
@@ -1936,10 +2138,10 @@
       <c r="E9" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="F9" s="16">
+      <c r="F9" s="17">
         <v>1</v>
       </c>
-      <c r="G9" s="21" t="s">
+      <c r="G9" s="22" t="s">
         <v>28</v>
       </c>
       <c r="H9" s="14" t="s">
@@ -1971,10 +2173,10 @@
     <row r="10" ht="42.75">
       <c r="A10" s="1"/>
       <c r="B10" s="15"/>
-      <c r="C10" s="15"/>
-      <c r="D10" s="15"/>
-      <c r="E10" s="15"/>
-      <c r="F10" s="16">
+      <c r="C10" s="16"/>
+      <c r="D10" s="16"/>
+      <c r="E10" s="16"/>
+      <c r="F10" s="17">
         <v>2</v>
       </c>
       <c r="G10" s="14" t="s">
@@ -2008,15 +2210,15 @@
     </row>
     <row r="11" ht="14.25" customHeight="1">
       <c r="A11" s="1"/>
-      <c r="B11" s="17"/>
-      <c r="C11" s="18"/>
-      <c r="D11" s="18"/>
-      <c r="E11" s="18"/>
-      <c r="F11" s="19"/>
-      <c r="G11" s="20"/>
-      <c r="H11" s="20"/>
-      <c r="I11" s="20"/>
-      <c r="J11" s="20"/>
+      <c r="B11" s="23"/>
+      <c r="C11" s="19"/>
+      <c r="D11" s="19"/>
+      <c r="E11" s="19"/>
+      <c r="F11" s="20"/>
+      <c r="G11" s="21"/>
+      <c r="H11" s="21"/>
+      <c r="I11" s="21"/>
+      <c r="J11" s="21"/>
       <c r="K11" s="1"/>
       <c r="L11" s="1"/>
       <c r="M11" s="1"/>
@@ -2036,7 +2238,7 @@
     </row>
     <row r="12" ht="46.5" customHeight="1">
       <c r="A12" s="1"/>
-      <c r="B12" s="11" t="s">
+      <c r="B12" s="24" t="s">
         <v>36</v>
       </c>
       <c r="C12" s="12" t="s">
@@ -2048,7 +2250,7 @@
       <c r="E12" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="F12" s="16">
+      <c r="F12" s="17">
         <v>1</v>
       </c>
       <c r="G12" s="14" t="s">
@@ -2082,11 +2284,11 @@
     </row>
     <row r="13" ht="42.75">
       <c r="A13" s="1"/>
-      <c r="B13" s="15"/>
-      <c r="C13" s="15"/>
-      <c r="D13" s="15"/>
-      <c r="E13" s="15"/>
-      <c r="F13" s="16">
+      <c r="B13" s="25"/>
+      <c r="C13" s="16"/>
+      <c r="D13" s="16"/>
+      <c r="E13" s="16"/>
+      <c r="F13" s="17">
         <v>2</v>
       </c>
       <c r="G13" s="14" t="s">
@@ -2120,15 +2322,15 @@
     </row>
     <row r="14" ht="14.25" customHeight="1">
       <c r="A14" s="1"/>
-      <c r="B14" s="19"/>
-      <c r="C14" s="20"/>
-      <c r="D14" s="20"/>
-      <c r="E14" s="20"/>
-      <c r="F14" s="19"/>
-      <c r="G14" s="20"/>
-      <c r="H14" s="20"/>
-      <c r="I14" s="20"/>
-      <c r="J14" s="20"/>
+      <c r="B14" s="26"/>
+      <c r="C14" s="21"/>
+      <c r="D14" s="21"/>
+      <c r="E14" s="21"/>
+      <c r="F14" s="20"/>
+      <c r="G14" s="21"/>
+      <c r="H14" s="21"/>
+      <c r="I14" s="21"/>
+      <c r="J14" s="21"/>
       <c r="K14" s="1"/>
       <c r="L14" s="1"/>
       <c r="M14" s="1"/>
@@ -2148,7 +2350,7 @@
     </row>
     <row r="15" ht="42.75">
       <c r="A15" s="1"/>
-      <c r="B15" s="11" t="s">
+      <c r="B15" s="24" t="s">
         <v>47</v>
       </c>
       <c r="C15" s="12" t="s">
@@ -2160,7 +2362,7 @@
       <c r="E15" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="F15" s="16">
+      <c r="F15" s="17">
         <v>1</v>
       </c>
       <c r="G15" s="14" t="s">
@@ -2194,11 +2396,11 @@
     </row>
     <row r="16" ht="42.75">
       <c r="A16" s="1"/>
-      <c r="B16" s="22"/>
-      <c r="C16" s="22"/>
-      <c r="D16" s="22"/>
-      <c r="E16" s="22"/>
-      <c r="F16" s="16">
+      <c r="B16" s="27"/>
+      <c r="C16" s="28"/>
+      <c r="D16" s="28"/>
+      <c r="E16" s="28"/>
+      <c r="F16" s="17">
         <v>2</v>
       </c>
       <c r="G16" s="14" t="s">
@@ -2232,11 +2434,11 @@
     </row>
     <row r="17" ht="36.5" customHeight="1">
       <c r="A17" s="1"/>
-      <c r="B17" s="22"/>
-      <c r="C17" s="22"/>
-      <c r="D17" s="22"/>
-      <c r="E17" s="22"/>
-      <c r="F17" s="11">
+      <c r="B17" s="27"/>
+      <c r="C17" s="28"/>
+      <c r="D17" s="28"/>
+      <c r="E17" s="28"/>
+      <c r="F17" s="29">
         <v>3</v>
       </c>
       <c r="G17" s="12" t="s">
@@ -2270,15 +2472,15 @@
     </row>
     <row r="18" ht="15">
       <c r="A18" s="1"/>
-      <c r="B18" s="15"/>
-      <c r="C18" s="15"/>
-      <c r="D18" s="15"/>
-      <c r="E18" s="15"/>
-      <c r="F18" s="15"/>
-      <c r="G18" s="15"/>
-      <c r="H18" s="15"/>
-      <c r="I18" s="15"/>
-      <c r="J18" s="15"/>
+      <c r="B18" s="25"/>
+      <c r="C18" s="16"/>
+      <c r="D18" s="16"/>
+      <c r="E18" s="16"/>
+      <c r="F18" s="16"/>
+      <c r="G18" s="16"/>
+      <c r="H18" s="16"/>
+      <c r="I18" s="16"/>
+      <c r="J18" s="16"/>
       <c r="K18" s="1"/>
       <c r="L18" s="1"/>
       <c r="M18" s="1"/>
@@ -2298,15 +2500,15 @@
     </row>
     <row r="19" ht="15">
       <c r="A19" s="1"/>
-      <c r="B19" s="23"/>
-      <c r="C19" s="24"/>
-      <c r="D19" s="25"/>
-      <c r="E19" s="24"/>
-      <c r="F19" s="24"/>
-      <c r="G19" s="25"/>
-      <c r="H19" s="25"/>
-      <c r="I19" s="25"/>
-      <c r="J19" s="25"/>
+      <c r="B19" s="30"/>
+      <c r="C19" s="31"/>
+      <c r="D19" s="32"/>
+      <c r="E19" s="31"/>
+      <c r="F19" s="31"/>
+      <c r="G19" s="32"/>
+      <c r="H19" s="32"/>
+      <c r="I19" s="32"/>
+      <c r="J19" s="32"/>
       <c r="K19" s="1"/>
       <c r="L19" s="1"/>
       <c r="M19" s="1"/>
@@ -2324,34 +2526,34 @@
       <c r="Y19" s="1"/>
       <c r="Z19" s="1"/>
     </row>
-    <row r="20" ht="42.75">
+    <row r="20" ht="69" customHeight="1">
       <c r="A20" s="1"/>
-      <c r="B20" s="26" t="s">
+      <c r="B20" s="33" t="s">
         <v>63</v>
       </c>
-      <c r="C20" s="26" t="s">
-        <v>25</v>
-      </c>
-      <c r="D20" s="26" t="s">
+      <c r="C20" s="34" t="s">
         <v>64</v>
       </c>
-      <c r="E20" s="26" t="s">
+      <c r="D20" s="34" t="s">
         <v>65</v>
       </c>
-      <c r="F20" s="16">
+      <c r="E20" s="34" t="s">
+        <v>66</v>
+      </c>
+      <c r="F20" s="13">
         <v>1</v>
       </c>
-      <c r="G20" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="H20" s="14" t="s">
+      <c r="G20" s="35" t="s">
         <v>67</v>
       </c>
-      <c r="I20" s="14" t="s">
+      <c r="H20" s="35" t="s">
         <v>68</v>
       </c>
-      <c r="J20" s="14" t="s">
+      <c r="I20" s="35" t="s">
         <v>69</v>
+      </c>
+      <c r="J20" s="35" t="s">
+        <v>70</v>
       </c>
       <c r="K20" s="1"/>
       <c r="L20" s="1"/>
@@ -2370,27 +2572,17 @@
       <c r="Y20" s="1"/>
       <c r="Z20" s="1"/>
     </row>
-    <row r="21" ht="42.75">
+    <row r="21" ht="13.5" customHeight="1">
       <c r="A21" s="1"/>
-      <c r="B21" s="27"/>
-      <c r="C21" s="27"/>
-      <c r="D21" s="27"/>
-      <c r="E21" s="27"/>
-      <c r="F21" s="16">
-        <v>2</v>
-      </c>
-      <c r="G21" s="14" t="s">
-        <v>70</v>
-      </c>
-      <c r="H21" s="14" t="s">
-        <v>71</v>
-      </c>
-      <c r="I21" s="14" t="s">
-        <v>72</v>
-      </c>
-      <c r="J21" s="14" t="s">
-        <v>73</v>
-      </c>
+      <c r="B21" s="30"/>
+      <c r="C21" s="31"/>
+      <c r="D21" s="32"/>
+      <c r="E21" s="31"/>
+      <c r="F21" s="31"/>
+      <c r="G21" s="32"/>
+      <c r="H21" s="32"/>
+      <c r="I21" s="32"/>
+      <c r="J21" s="32"/>
       <c r="K21" s="1"/>
       <c r="L21" s="1"/>
       <c r="M21" s="1"/>
@@ -2410,23 +2602,31 @@
     </row>
     <row r="22" ht="42.75">
       <c r="A22" s="1"/>
-      <c r="B22" s="28"/>
-      <c r="C22" s="28"/>
-      <c r="D22" s="28"/>
-      <c r="E22" s="28"/>
-      <c r="F22" s="16">
-        <v>3</v>
+      <c r="B22" s="36" t="s">
+        <v>71</v>
       </c>
-      <c r="G22" s="29" t="s">
+      <c r="C22" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="D22" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="E22" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="F22" s="17">
+        <v>1</v>
+      </c>
+      <c r="G22" s="14" t="s">
         <v>74</v>
       </c>
-      <c r="H22" s="29" t="s">
+      <c r="H22" s="14" t="s">
         <v>75</v>
       </c>
-      <c r="I22" s="29" t="s">
+      <c r="I22" s="14" t="s">
         <v>76</v>
       </c>
-      <c r="J22" s="29" t="s">
+      <c r="J22" s="14" t="s">
         <v>77</v>
       </c>
       <c r="K22" s="1"/>
@@ -2446,17 +2646,27 @@
       <c r="Y22" s="1"/>
       <c r="Z22" s="1"/>
     </row>
-    <row r="23" ht="15">
+    <row r="23" ht="42.75">
       <c r="A23" s="1"/>
-      <c r="B23" s="23"/>
-      <c r="C23" s="24"/>
-      <c r="D23" s="25"/>
-      <c r="E23" s="24"/>
-      <c r="F23" s="24"/>
-      <c r="G23" s="25"/>
-      <c r="H23" s="25"/>
-      <c r="I23" s="25"/>
-      <c r="J23" s="25"/>
+      <c r="B23" s="36"/>
+      <c r="C23" s="16"/>
+      <c r="D23" s="16"/>
+      <c r="E23" s="16"/>
+      <c r="F23" s="17">
+        <v>2</v>
+      </c>
+      <c r="G23" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="H23" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="I23" s="14" t="s">
+        <v>80</v>
+      </c>
+      <c r="J23" s="14" t="s">
+        <v>81</v>
+      </c>
       <c r="K23" s="1"/>
       <c r="L23" s="1"/>
       <c r="M23" s="1"/>
@@ -2474,35 +2684,17 @@
       <c r="Y23" s="1"/>
       <c r="Z23" s="1"/>
     </row>
-    <row r="24" ht="28.5">
+    <row r="24" ht="17.5" customHeight="1">
       <c r="A24" s="1"/>
-      <c r="B24" s="11" t="s">
-        <v>78</v>
-      </c>
-      <c r="C24" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="D24" s="12" t="s">
-        <v>79</v>
-      </c>
-      <c r="E24" s="12" t="s">
-        <v>80</v>
-      </c>
-      <c r="F24" s="16">
-        <v>1</v>
-      </c>
-      <c r="G24" s="14" t="s">
-        <v>81</v>
-      </c>
-      <c r="H24" s="14" t="s">
-        <v>82</v>
-      </c>
-      <c r="I24" s="14" t="s">
-        <v>83</v>
-      </c>
-      <c r="J24" s="14" t="s">
-        <v>84</v>
-      </c>
+      <c r="B24" s="30"/>
+      <c r="C24" s="31"/>
+      <c r="D24" s="32"/>
+      <c r="E24" s="31"/>
+      <c r="F24" s="31"/>
+      <c r="G24" s="32"/>
+      <c r="H24" s="32"/>
+      <c r="I24" s="32"/>
+      <c r="J24" s="32"/>
       <c r="K24" s="1"/>
       <c r="L24" s="1"/>
       <c r="M24" s="1"/>
@@ -2522,24 +2714,32 @@
     </row>
     <row r="25" ht="42.75">
       <c r="A25" s="1"/>
-      <c r="B25" s="15"/>
-      <c r="C25" s="15"/>
-      <c r="D25" s="15"/>
-      <c r="E25" s="15"/>
-      <c r="F25" s="16">
-        <v>2</v>
+      <c r="B25" s="37" t="s">
+        <v>82</v>
+      </c>
+      <c r="C25" s="38" t="s">
+        <v>83</v>
+      </c>
+      <c r="D25" s="38" t="s">
+        <v>84</v>
+      </c>
+      <c r="E25" s="38" t="s">
+        <v>85</v>
+      </c>
+      <c r="F25" s="17">
+        <v>1</v>
       </c>
       <c r="G25" s="14" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H25" s="14" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="I25" s="14" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J25" s="14" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="K25" s="1"/>
       <c r="L25" s="1"/>
@@ -2558,17 +2758,27 @@
       <c r="Y25" s="1"/>
       <c r="Z25" s="1"/>
     </row>
-    <row r="26" ht="15">
+    <row r="26" ht="80.5" customHeight="1">
       <c r="A26" s="1"/>
-      <c r="B26" s="23"/>
-      <c r="C26" s="24"/>
-      <c r="D26" s="25"/>
-      <c r="E26" s="24"/>
-      <c r="F26" s="24"/>
-      <c r="G26" s="25"/>
-      <c r="H26" s="25"/>
-      <c r="I26" s="25"/>
-      <c r="J26" s="25"/>
+      <c r="B26" s="37"/>
+      <c r="C26" s="38"/>
+      <c r="D26" s="38"/>
+      <c r="E26" s="38"/>
+      <c r="F26" s="13">
+        <v>2</v>
+      </c>
+      <c r="G26" s="35" t="s">
+        <v>90</v>
+      </c>
+      <c r="H26" s="35" t="s">
+        <v>91</v>
+      </c>
+      <c r="I26" s="35" t="s">
+        <v>92</v>
+      </c>
+      <c r="J26" s="35" t="s">
+        <v>93</v>
+      </c>
       <c r="K26" s="1"/>
       <c r="L26" s="1"/>
       <c r="M26" s="1"/>
@@ -2586,35 +2796,17 @@
       <c r="Y26" s="1"/>
       <c r="Z26" s="1"/>
     </row>
-    <row r="27" ht="42.75">
+    <row r="27" ht="15">
       <c r="A27" s="1"/>
-      <c r="B27" s="11" t="s">
-        <v>89</v>
-      </c>
-      <c r="C27" s="12" t="s">
-        <v>48</v>
-      </c>
-      <c r="D27" s="12" t="s">
-        <v>90</v>
-      </c>
-      <c r="E27" s="12" t="s">
-        <v>91</v>
-      </c>
-      <c r="F27" s="16">
-        <v>1</v>
-      </c>
-      <c r="G27" s="14" t="s">
-        <v>92</v>
-      </c>
-      <c r="H27" s="14" t="s">
-        <v>93</v>
-      </c>
-      <c r="I27" s="14" t="s">
-        <v>94</v>
-      </c>
-      <c r="J27" s="14" t="s">
-        <v>95</v>
-      </c>
+      <c r="B27" s="39"/>
+      <c r="C27" s="40"/>
+      <c r="D27" s="40"/>
+      <c r="E27" s="40"/>
+      <c r="F27" s="40"/>
+      <c r="G27" s="40"/>
+      <c r="H27" s="40"/>
+      <c r="I27" s="40"/>
+      <c r="J27" s="40"/>
       <c r="K27" s="1"/>
       <c r="L27" s="1"/>
       <c r="M27" s="1"/>
@@ -2632,26 +2824,34 @@
       <c r="Y27" s="1"/>
       <c r="Z27" s="1"/>
     </row>
-    <row r="28" ht="42.75">
+    <row r="28" ht="57">
       <c r="A28" s="1"/>
-      <c r="B28" s="15"/>
-      <c r="C28" s="15"/>
-      <c r="D28" s="15"/>
-      <c r="E28" s="15"/>
-      <c r="F28" s="16">
-        <v>2</v>
+      <c r="B28" s="36" t="s">
+        <v>94</v>
       </c>
-      <c r="G28" s="14" t="s">
+      <c r="C28" s="41" t="s">
+        <v>13</v>
+      </c>
+      <c r="D28" s="41" t="s">
+        <v>95</v>
+      </c>
+      <c r="E28" s="41" t="s">
         <v>96</v>
       </c>
-      <c r="H28" s="14" t="s">
+      <c r="F28" s="13">
+        <v>1</v>
+      </c>
+      <c r="G28" s="35" t="s">
         <v>97</v>
       </c>
-      <c r="I28" s="14" t="s">
+      <c r="H28" s="35" t="s">
         <v>98</v>
       </c>
-      <c r="J28" s="14" t="s">
+      <c r="I28" s="35" t="s">
         <v>99</v>
+      </c>
+      <c r="J28" s="35" t="s">
+        <v>100</v>
       </c>
       <c r="K28" s="1"/>
       <c r="L28" s="1"/>
@@ -2670,17 +2870,27 @@
       <c r="Y28" s="1"/>
       <c r="Z28" s="1"/>
     </row>
-    <row r="29" ht="14.25" customHeight="1">
+    <row r="29" ht="42.75">
       <c r="A29" s="1"/>
-      <c r="B29" s="23"/>
-      <c r="C29" s="24"/>
-      <c r="D29" s="25"/>
-      <c r="E29" s="24"/>
-      <c r="F29" s="24"/>
-      <c r="G29" s="25"/>
-      <c r="H29" s="25"/>
-      <c r="I29" s="25"/>
-      <c r="J29" s="25"/>
+      <c r="B29" s="36"/>
+      <c r="C29" s="41"/>
+      <c r="D29" s="41"/>
+      <c r="E29" s="41"/>
+      <c r="F29" s="13">
+        <v>2</v>
+      </c>
+      <c r="G29" s="35" t="s">
+        <v>101</v>
+      </c>
+      <c r="H29" s="35" t="s">
+        <v>102</v>
+      </c>
+      <c r="I29" s="35" t="s">
+        <v>103</v>
+      </c>
+      <c r="J29" s="35" t="s">
+        <v>104</v>
+      </c>
       <c r="K29" s="1"/>
       <c r="L29" s="1"/>
       <c r="M29" s="1"/>
@@ -2698,35 +2908,17 @@
       <c r="Y29" s="1"/>
       <c r="Z29" s="1"/>
     </row>
-    <row r="30" ht="42.75">
+    <row r="30" ht="15">
       <c r="A30" s="1"/>
-      <c r="B30" s="11" t="s">
-        <v>100</v>
-      </c>
-      <c r="C30" s="12" t="s">
-        <v>101</v>
-      </c>
-      <c r="D30" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="E30" s="12" t="s">
-        <v>103</v>
-      </c>
-      <c r="F30" s="16">
-        <v>1</v>
-      </c>
-      <c r="G30" s="14" t="s">
-        <v>104</v>
-      </c>
-      <c r="H30" s="14" t="s">
-        <v>105</v>
-      </c>
-      <c r="I30" s="14" t="s">
-        <v>106</v>
-      </c>
-      <c r="J30" s="14" t="s">
-        <v>107</v>
-      </c>
+      <c r="B30" s="40"/>
+      <c r="C30" s="42"/>
+      <c r="D30" s="43"/>
+      <c r="E30" s="42"/>
+      <c r="F30" s="31"/>
+      <c r="G30" s="32"/>
+      <c r="H30" s="32"/>
+      <c r="I30" s="32"/>
+      <c r="J30" s="32"/>
       <c r="K30" s="1"/>
       <c r="L30" s="1"/>
       <c r="M30" s="1"/>
@@ -2746,12 +2938,20 @@
     </row>
     <row r="31" ht="42.75">
       <c r="A31" s="1"/>
-      <c r="B31" s="22"/>
-      <c r="C31" s="22"/>
-      <c r="D31" s="22"/>
-      <c r="E31" s="22"/>
-      <c r="F31" s="16">
-        <v>2</v>
+      <c r="B31" s="44" t="s">
+        <v>105</v>
+      </c>
+      <c r="C31" s="45" t="s">
+        <v>25</v>
+      </c>
+      <c r="D31" s="45" t="s">
+        <v>106</v>
+      </c>
+      <c r="E31" s="45" t="s">
+        <v>107</v>
+      </c>
+      <c r="F31" s="17">
+        <v>1</v>
       </c>
       <c r="G31" s="14" t="s">
         <v>108</v>
@@ -2782,14 +2982,14 @@
       <c r="Y31" s="1"/>
       <c r="Z31" s="1"/>
     </row>
-    <row r="32" ht="28.5">
+    <row r="32" ht="42.75">
       <c r="A32" s="1"/>
-      <c r="B32" s="15"/>
-      <c r="C32" s="15"/>
-      <c r="D32" s="15"/>
-      <c r="E32" s="15"/>
-      <c r="F32" s="16">
-        <v>3</v>
+      <c r="B32" s="46"/>
+      <c r="C32" s="47"/>
+      <c r="D32" s="47"/>
+      <c r="E32" s="47"/>
+      <c r="F32" s="17">
+        <v>2</v>
       </c>
       <c r="G32" s="14" t="s">
         <v>112</v>
@@ -2820,17 +3020,27 @@
       <c r="Y32" s="1"/>
       <c r="Z32" s="1"/>
     </row>
-    <row r="33" ht="14.25" customHeight="1">
+    <row r="33" ht="42.75">
       <c r="A33" s="1"/>
-      <c r="B33" s="23"/>
-      <c r="C33" s="24"/>
-      <c r="D33" s="25"/>
-      <c r="E33" s="24"/>
-      <c r="F33" s="24"/>
-      <c r="G33" s="25"/>
-      <c r="H33" s="25"/>
-      <c r="I33" s="25"/>
-      <c r="J33" s="25"/>
+      <c r="B33" s="48"/>
+      <c r="C33" s="49"/>
+      <c r="D33" s="49"/>
+      <c r="E33" s="49"/>
+      <c r="F33" s="17">
+        <v>3</v>
+      </c>
+      <c r="G33" s="50" t="s">
+        <v>116</v>
+      </c>
+      <c r="H33" s="50" t="s">
+        <v>117</v>
+      </c>
+      <c r="I33" s="50" t="s">
+        <v>118</v>
+      </c>
+      <c r="J33" s="50" t="s">
+        <v>119</v>
+      </c>
       <c r="K33" s="1"/>
       <c r="L33" s="1"/>
       <c r="M33" s="1"/>
@@ -2848,35 +3058,17 @@
       <c r="Y33" s="1"/>
       <c r="Z33" s="1"/>
     </row>
-    <row r="34" ht="42.75">
+    <row r="34" ht="15">
       <c r="A34" s="1"/>
-      <c r="B34" s="11" t="s">
-        <v>116</v>
-      </c>
-      <c r="C34" s="12" t="s">
-        <v>48</v>
-      </c>
-      <c r="D34" s="12" t="s">
-        <v>117</v>
-      </c>
-      <c r="E34" s="12" t="s">
-        <v>118</v>
-      </c>
-      <c r="F34" s="16">
-        <v>1</v>
-      </c>
-      <c r="G34" s="14" t="s">
-        <v>119</v>
-      </c>
-      <c r="H34" s="14" t="s">
-        <v>120</v>
-      </c>
-      <c r="I34" s="14" t="s">
-        <v>121</v>
-      </c>
-      <c r="J34" s="14" t="s">
-        <v>122</v>
-      </c>
+      <c r="B34" s="51"/>
+      <c r="C34" s="31"/>
+      <c r="D34" s="32"/>
+      <c r="E34" s="31"/>
+      <c r="F34" s="31"/>
+      <c r="G34" s="32"/>
+      <c r="H34" s="32"/>
+      <c r="I34" s="32"/>
+      <c r="J34" s="32"/>
       <c r="K34" s="1"/>
       <c r="L34" s="1"/>
       <c r="M34" s="1"/>
@@ -2894,14 +3086,22 @@
       <c r="Y34" s="1"/>
       <c r="Z34" s="1"/>
     </row>
-    <row r="35" ht="42.75">
+    <row r="35" ht="28.5">
       <c r="A35" s="1"/>
-      <c r="B35" s="15"/>
-      <c r="C35" s="15"/>
-      <c r="D35" s="15"/>
-      <c r="E35" s="15"/>
-      <c r="F35" s="16">
-        <v>2</v>
+      <c r="B35" s="52" t="s">
+        <v>120</v>
+      </c>
+      <c r="C35" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="D35" s="12" t="s">
+        <v>121</v>
+      </c>
+      <c r="E35" s="12" t="s">
+        <v>122</v>
+      </c>
+      <c r="F35" s="17">
+        <v>1</v>
       </c>
       <c r="G35" s="14" t="s">
         <v>123</v>
@@ -2932,17 +3132,27 @@
       <c r="Y35" s="1"/>
       <c r="Z35" s="1"/>
     </row>
-    <row r="36" ht="14.25" customHeight="1">
+    <row r="36" ht="42.75">
       <c r="A36" s="1"/>
-      <c r="B36" s="23"/>
-      <c r="C36" s="24"/>
-      <c r="D36" s="25"/>
-      <c r="E36" s="24"/>
-      <c r="F36" s="24"/>
-      <c r="G36" s="25"/>
-      <c r="H36" s="25"/>
-      <c r="I36" s="25"/>
-      <c r="J36" s="25"/>
+      <c r="B36" s="53"/>
+      <c r="C36" s="16"/>
+      <c r="D36" s="16"/>
+      <c r="E36" s="16"/>
+      <c r="F36" s="17">
+        <v>2</v>
+      </c>
+      <c r="G36" s="14" t="s">
+        <v>127</v>
+      </c>
+      <c r="H36" s="14" t="s">
+        <v>128</v>
+      </c>
+      <c r="I36" s="14" t="s">
+        <v>129</v>
+      </c>
+      <c r="J36" s="14" t="s">
+        <v>130</v>
+      </c>
       <c r="K36" s="1"/>
       <c r="L36" s="1"/>
       <c r="M36" s="1"/>
@@ -2960,35 +3170,17 @@
       <c r="Y36" s="1"/>
       <c r="Z36" s="1"/>
     </row>
-    <row r="37" ht="42.75">
+    <row r="37" ht="15">
       <c r="A37" s="1"/>
-      <c r="B37" s="30" t="s">
-        <v>127</v>
-      </c>
-      <c r="C37" s="31" t="s">
-        <v>48</v>
-      </c>
-      <c r="D37" s="31" t="s">
-        <v>128</v>
-      </c>
-      <c r="E37" s="31" t="s">
-        <v>129</v>
-      </c>
-      <c r="F37" s="32">
-        <v>1</v>
-      </c>
-      <c r="G37" s="33" t="s">
-        <v>130</v>
-      </c>
-      <c r="H37" s="33" t="s">
-        <v>131</v>
-      </c>
-      <c r="I37" s="33" t="s">
-        <v>132</v>
-      </c>
-      <c r="J37" s="33" t="s">
-        <v>133</v>
-      </c>
+      <c r="B37" s="51"/>
+      <c r="C37" s="31"/>
+      <c r="D37" s="32"/>
+      <c r="E37" s="31"/>
+      <c r="F37" s="31"/>
+      <c r="G37" s="32"/>
+      <c r="H37" s="32"/>
+      <c r="I37" s="32"/>
+      <c r="J37" s="32"/>
       <c r="K37" s="1"/>
       <c r="L37" s="1"/>
       <c r="M37" s="1"/>
@@ -3008,23 +3200,31 @@
     </row>
     <row r="38" ht="42.75">
       <c r="A38" s="1"/>
-      <c r="B38" s="15"/>
-      <c r="C38" s="15"/>
-      <c r="D38" s="15"/>
-      <c r="E38" s="15"/>
-      <c r="F38" s="32">
-        <v>2</v>
+      <c r="B38" s="52" t="s">
+        <v>131</v>
       </c>
-      <c r="G38" s="33" t="s">
+      <c r="C38" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="D38" s="12" t="s">
+        <v>132</v>
+      </c>
+      <c r="E38" s="12" t="s">
+        <v>133</v>
+      </c>
+      <c r="F38" s="17">
+        <v>1</v>
+      </c>
+      <c r="G38" s="14" t="s">
         <v>134</v>
       </c>
-      <c r="H38" s="33" t="s">
+      <c r="H38" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="I38" s="33" t="s">
+      <c r="I38" s="14" t="s">
         <v>136</v>
       </c>
-      <c r="J38" s="33" t="s">
+      <c r="J38" s="14" t="s">
         <v>137</v>
       </c>
       <c r="K38" s="1"/>
@@ -3044,17 +3244,27 @@
       <c r="Y38" s="1"/>
       <c r="Z38" s="1"/>
     </row>
-    <row r="39" ht="14.25" customHeight="1">
+    <row r="39" ht="42.75">
       <c r="A39" s="1"/>
-      <c r="B39" s="23"/>
-      <c r="C39" s="24"/>
-      <c r="D39" s="25"/>
-      <c r="E39" s="24"/>
-      <c r="F39" s="24"/>
-      <c r="G39" s="25"/>
-      <c r="H39" s="25"/>
-      <c r="I39" s="25"/>
-      <c r="J39" s="25"/>
+      <c r="B39" s="53"/>
+      <c r="C39" s="16"/>
+      <c r="D39" s="16"/>
+      <c r="E39" s="16"/>
+      <c r="F39" s="17">
+        <v>2</v>
+      </c>
+      <c r="G39" s="14" t="s">
+        <v>138</v>
+      </c>
+      <c r="H39" s="14" t="s">
+        <v>139</v>
+      </c>
+      <c r="I39" s="14" t="s">
+        <v>140</v>
+      </c>
+      <c r="J39" s="14" t="s">
+        <v>141</v>
+      </c>
       <c r="K39" s="1"/>
       <c r="L39" s="1"/>
       <c r="M39" s="1"/>
@@ -3072,35 +3282,17 @@
       <c r="Y39" s="1"/>
       <c r="Z39" s="1"/>
     </row>
-    <row r="40" ht="42.75">
+    <row r="40" ht="14.25" customHeight="1">
       <c r="A40" s="1"/>
-      <c r="B40" s="11" t="s">
-        <v>138</v>
-      </c>
-      <c r="C40" s="12" t="s">
-        <v>48</v>
-      </c>
-      <c r="D40" s="12" t="s">
-        <v>139</v>
-      </c>
-      <c r="E40" s="12" t="s">
-        <v>140</v>
-      </c>
-      <c r="F40" s="16">
-        <v>1</v>
-      </c>
-      <c r="G40" s="14" t="s">
-        <v>141</v>
-      </c>
-      <c r="H40" s="14" t="s">
-        <v>142</v>
-      </c>
-      <c r="I40" s="14" t="s">
-        <v>143</v>
-      </c>
-      <c r="J40" s="14" t="s">
-        <v>144</v>
-      </c>
+      <c r="B40" s="54"/>
+      <c r="C40" s="31"/>
+      <c r="D40" s="32"/>
+      <c r="E40" s="31"/>
+      <c r="F40" s="31"/>
+      <c r="G40" s="32"/>
+      <c r="H40" s="32"/>
+      <c r="I40" s="32"/>
+      <c r="J40" s="32"/>
       <c r="K40" s="1"/>
       <c r="L40" s="1"/>
       <c r="M40" s="1"/>
@@ -3120,24 +3312,32 @@
     </row>
     <row r="41" ht="42.75">
       <c r="A41" s="1"/>
-      <c r="B41" s="15"/>
-      <c r="C41" s="15"/>
-      <c r="D41" s="15"/>
-      <c r="E41" s="15"/>
-      <c r="F41" s="16">
-        <v>2</v>
+      <c r="B41" s="55" t="s">
+        <v>142</v>
+      </c>
+      <c r="C41" s="12" t="s">
+        <v>143</v>
+      </c>
+      <c r="D41" s="12" t="s">
+        <v>144</v>
+      </c>
+      <c r="E41" s="12" t="s">
+        <v>145</v>
+      </c>
+      <c r="F41" s="17">
+        <v>1</v>
       </c>
       <c r="G41" s="14" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H41" s="14" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="I41" s="14" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="J41" s="14" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="K41" s="1"/>
       <c r="L41" s="1"/>
@@ -3156,17 +3356,27 @@
       <c r="Y41" s="1"/>
       <c r="Z41" s="1"/>
     </row>
-    <row r="42" ht="15">
+    <row r="42" ht="42.75">
       <c r="A42" s="1"/>
-      <c r="B42" s="23"/>
-      <c r="C42" s="24"/>
-      <c r="D42" s="25"/>
-      <c r="E42" s="24"/>
-      <c r="F42" s="24"/>
-      <c r="G42" s="25"/>
-      <c r="H42" s="25"/>
-      <c r="I42" s="25"/>
-      <c r="J42" s="25"/>
+      <c r="B42" s="56"/>
+      <c r="C42" s="28"/>
+      <c r="D42" s="28"/>
+      <c r="E42" s="28"/>
+      <c r="F42" s="17">
+        <v>2</v>
+      </c>
+      <c r="G42" s="14" t="s">
+        <v>150</v>
+      </c>
+      <c r="H42" s="14" t="s">
+        <v>151</v>
+      </c>
+      <c r="I42" s="14" t="s">
+        <v>152</v>
+      </c>
+      <c r="J42" s="14" t="s">
+        <v>153</v>
+      </c>
       <c r="K42" s="1"/>
       <c r="L42" s="1"/>
       <c r="M42" s="1"/>
@@ -3184,34 +3394,26 @@
       <c r="Y42" s="1"/>
       <c r="Z42" s="1"/>
     </row>
-    <row r="43" ht="42.75">
+    <row r="43" ht="28.5">
       <c r="A43" s="1"/>
-      <c r="B43" s="11" t="s">
-        <v>149</v>
-      </c>
-      <c r="C43" s="12" t="s">
-        <v>48</v>
-      </c>
-      <c r="D43" s="12" t="s">
-        <v>150</v>
-      </c>
-      <c r="E43" s="12" t="s">
-        <v>151</v>
-      </c>
-      <c r="F43" s="16">
-        <v>1</v>
+      <c r="B43" s="57"/>
+      <c r="C43" s="16"/>
+      <c r="D43" s="16"/>
+      <c r="E43" s="16"/>
+      <c r="F43" s="17">
+        <v>3</v>
       </c>
       <c r="G43" s="14" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="H43" s="14" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="I43" s="14" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="J43" s="14" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="K43" s="1"/>
       <c r="L43" s="1"/>
@@ -3230,27 +3432,17 @@
       <c r="Y43" s="1"/>
       <c r="Z43" s="1"/>
     </row>
-    <row r="44" ht="42.75">
+    <row r="44" ht="14.25" customHeight="1">
       <c r="A44" s="1"/>
-      <c r="B44" s="15"/>
-      <c r="C44" s="15"/>
-      <c r="D44" s="15"/>
-      <c r="E44" s="15"/>
-      <c r="F44" s="16">
-        <v>2</v>
-      </c>
-      <c r="G44" s="14" t="s">
-        <v>156</v>
-      </c>
-      <c r="H44" s="14" t="s">
-        <v>157</v>
-      </c>
-      <c r="I44" s="14" t="s">
-        <v>158</v>
-      </c>
-      <c r="J44" s="14" t="s">
-        <v>159</v>
-      </c>
+      <c r="B44" s="58"/>
+      <c r="C44" s="31"/>
+      <c r="D44" s="32"/>
+      <c r="E44" s="31"/>
+      <c r="F44" s="31"/>
+      <c r="G44" s="32"/>
+      <c r="H44" s="32"/>
+      <c r="I44" s="32"/>
+      <c r="J44" s="32"/>
       <c r="K44" s="1"/>
       <c r="L44" s="1"/>
       <c r="M44" s="1"/>
@@ -3268,17 +3460,35 @@
       <c r="Y44" s="1"/>
       <c r="Z44" s="1"/>
     </row>
-    <row r="45" ht="14.25" customHeight="1">
+    <row r="45" ht="42.75">
       <c r="A45" s="1"/>
-      <c r="B45" s="23"/>
-      <c r="C45" s="24"/>
-      <c r="D45" s="25"/>
-      <c r="E45" s="24"/>
-      <c r="F45" s="24"/>
-      <c r="G45" s="25"/>
-      <c r="H45" s="25"/>
-      <c r="I45" s="25"/>
-      <c r="J45" s="25"/>
+      <c r="B45" s="55" t="s">
+        <v>158</v>
+      </c>
+      <c r="C45" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="D45" s="12" t="s">
+        <v>159</v>
+      </c>
+      <c r="E45" s="12" t="s">
+        <v>160</v>
+      </c>
+      <c r="F45" s="17">
+        <v>1</v>
+      </c>
+      <c r="G45" s="14" t="s">
+        <v>161</v>
+      </c>
+      <c r="H45" s="14" t="s">
+        <v>162</v>
+      </c>
+      <c r="I45" s="14" t="s">
+        <v>163</v>
+      </c>
+      <c r="J45" s="14" t="s">
+        <v>164</v>
+      </c>
       <c r="K45" s="1"/>
       <c r="L45" s="1"/>
       <c r="M45" s="1"/>
@@ -3296,34 +3506,26 @@
       <c r="Y45" s="1"/>
       <c r="Z45" s="1"/>
     </row>
-    <row r="46" ht="57.75" customHeight="1">
+    <row r="46" ht="42.75">
       <c r="A46" s="1"/>
-      <c r="B46" s="11" t="s">
-        <v>160</v>
-      </c>
-      <c r="C46" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="D46" s="12" t="s">
-        <v>161</v>
-      </c>
-      <c r="E46" s="12" t="s">
-        <v>162</v>
-      </c>
-      <c r="F46" s="16">
-        <v>1</v>
+      <c r="B46" s="57"/>
+      <c r="C46" s="16"/>
+      <c r="D46" s="16"/>
+      <c r="E46" s="16"/>
+      <c r="F46" s="17">
+        <v>2</v>
       </c>
       <c r="G46" s="14" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="H46" s="14" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="I46" s="14" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="J46" s="14" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="K46" s="1"/>
       <c r="L46" s="1"/>
@@ -3342,27 +3544,17 @@
       <c r="Y46" s="1"/>
       <c r="Z46" s="1"/>
     </row>
-    <row r="47" ht="57" customHeight="1">
+    <row r="47" ht="14.25" customHeight="1">
       <c r="A47" s="1"/>
-      <c r="B47" s="15"/>
-      <c r="C47" s="15"/>
-      <c r="D47" s="15"/>
-      <c r="E47" s="15"/>
-      <c r="F47" s="16">
-        <v>2</v>
-      </c>
-      <c r="G47" s="14" t="s">
-        <v>167</v>
-      </c>
-      <c r="H47" s="14" t="s">
-        <v>168</v>
-      </c>
-      <c r="I47" s="14" t="s">
-        <v>169</v>
-      </c>
-      <c r="J47" s="14" t="s">
-        <v>170</v>
-      </c>
+      <c r="B47" s="58"/>
+      <c r="C47" s="31"/>
+      <c r="D47" s="32"/>
+      <c r="E47" s="31"/>
+      <c r="F47" s="31"/>
+      <c r="G47" s="32"/>
+      <c r="H47" s="32"/>
+      <c r="I47" s="32"/>
+      <c r="J47" s="32"/>
       <c r="K47" s="1"/>
       <c r="L47" s="1"/>
       <c r="M47" s="1"/>
@@ -3380,17 +3572,35 @@
       <c r="Y47" s="1"/>
       <c r="Z47" s="1"/>
     </row>
-    <row r="48" ht="14.25" customHeight="1">
+    <row r="48" ht="42.75">
       <c r="A48" s="1"/>
-      <c r="B48" s="23"/>
-      <c r="C48" s="24"/>
-      <c r="D48" s="25"/>
-      <c r="E48" s="24"/>
-      <c r="F48" s="24"/>
-      <c r="G48" s="25"/>
-      <c r="H48" s="25"/>
-      <c r="I48" s="25"/>
-      <c r="J48" s="25"/>
+      <c r="B48" s="55" t="s">
+        <v>169</v>
+      </c>
+      <c r="C48" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="D48" s="12" t="s">
+        <v>170</v>
+      </c>
+      <c r="E48" s="12" t="s">
+        <v>171</v>
+      </c>
+      <c r="F48" s="17">
+        <v>1</v>
+      </c>
+      <c r="G48" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="H48" s="14" t="s">
+        <v>173</v>
+      </c>
+      <c r="I48" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="J48" s="14" t="s">
+        <v>175</v>
+      </c>
       <c r="K48" s="1"/>
       <c r="L48" s="1"/>
       <c r="M48" s="1"/>
@@ -3408,34 +3618,26 @@
       <c r="Y48" s="1"/>
       <c r="Z48" s="1"/>
     </row>
-    <row r="49" ht="46.5" customHeight="1">
+    <row r="49" ht="42.75">
       <c r="A49" s="1"/>
-      <c r="B49" s="11" t="s">
-        <v>171</v>
-      </c>
-      <c r="C49" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="D49" s="12" t="s">
-        <v>172</v>
-      </c>
-      <c r="E49" s="12" t="s">
-        <v>173</v>
-      </c>
-      <c r="F49" s="16">
-        <v>1</v>
+      <c r="B49" s="57"/>
+      <c r="C49" s="16"/>
+      <c r="D49" s="16"/>
+      <c r="E49" s="16"/>
+      <c r="F49" s="17">
+        <v>2</v>
       </c>
       <c r="G49" s="14" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="H49" s="14" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="I49" s="14" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="J49" s="14" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="K49" s="1"/>
       <c r="L49" s="1"/>
@@ -3454,27 +3656,17 @@
       <c r="Y49" s="1"/>
       <c r="Z49" s="1"/>
     </row>
-    <row r="50" ht="40.5" customHeight="1">
+    <row r="50" ht="14.25" customHeight="1">
       <c r="A50" s="1"/>
-      <c r="B50" s="15"/>
-      <c r="C50" s="15"/>
-      <c r="D50" s="15"/>
-      <c r="E50" s="15"/>
-      <c r="F50" s="16">
-        <v>2</v>
-      </c>
-      <c r="G50" s="14" t="s">
-        <v>178</v>
-      </c>
-      <c r="H50" s="14" t="s">
-        <v>179</v>
-      </c>
-      <c r="I50" s="14" t="s">
-        <v>180</v>
-      </c>
-      <c r="J50" s="14" t="s">
-        <v>181</v>
-      </c>
+      <c r="B50" s="58"/>
+      <c r="C50" s="31"/>
+      <c r="D50" s="32"/>
+      <c r="E50" s="31"/>
+      <c r="F50" s="31"/>
+      <c r="G50" s="32"/>
+      <c r="H50" s="32"/>
+      <c r="I50" s="32"/>
+      <c r="J50" s="32"/>
       <c r="K50" s="1"/>
       <c r="L50" s="1"/>
       <c r="M50" s="1"/>
@@ -3492,17 +3684,35 @@
       <c r="Y50" s="1"/>
       <c r="Z50" s="1"/>
     </row>
-    <row r="51" ht="14.25" customHeight="1">
+    <row r="51" ht="57">
       <c r="A51" s="1"/>
-      <c r="B51" s="23"/>
-      <c r="C51" s="24"/>
-      <c r="D51" s="25"/>
-      <c r="E51" s="24"/>
-      <c r="F51" s="24"/>
-      <c r="G51" s="25"/>
-      <c r="H51" s="25"/>
-      <c r="I51" s="25"/>
-      <c r="J51" s="25"/>
+      <c r="B51" s="59" t="s">
+        <v>180</v>
+      </c>
+      <c r="C51" s="34" t="s">
+        <v>181</v>
+      </c>
+      <c r="D51" s="34" t="s">
+        <v>182</v>
+      </c>
+      <c r="E51" s="34" t="s">
+        <v>183</v>
+      </c>
+      <c r="F51" s="17">
+        <v>1</v>
+      </c>
+      <c r="G51" s="14" t="s">
+        <v>184</v>
+      </c>
+      <c r="H51" s="14" t="s">
+        <v>185</v>
+      </c>
+      <c r="I51" s="14" t="s">
+        <v>186</v>
+      </c>
+      <c r="J51" s="14" t="s">
+        <v>187</v>
+      </c>
       <c r="K51" s="1"/>
       <c r="L51" s="1"/>
       <c r="M51" s="1"/>
@@ -3520,34 +3730,26 @@
       <c r="Y51" s="1"/>
       <c r="Z51" s="1"/>
     </row>
-    <row r="52" ht="57">
+    <row r="52" ht="68.25" customHeight="1">
       <c r="A52" s="1"/>
-      <c r="B52" s="11" t="s">
-        <v>182</v>
-      </c>
-      <c r="C52" s="12" t="s">
-        <v>183</v>
-      </c>
-      <c r="D52" s="12" t="s">
-        <v>184</v>
-      </c>
-      <c r="E52" s="12" t="s">
-        <v>185</v>
-      </c>
-      <c r="F52" s="16">
-        <v>1</v>
+      <c r="B52" s="60"/>
+      <c r="C52" s="41"/>
+      <c r="D52" s="41"/>
+      <c r="E52" s="41"/>
+      <c r="F52" s="17">
+        <v>2</v>
       </c>
       <c r="G52" s="14" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="H52" s="14" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="I52" s="14" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="J52" s="14" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="K52" s="1"/>
       <c r="L52" s="1"/>
@@ -3566,26 +3768,26 @@
       <c r="Y52" s="1"/>
       <c r="Z52" s="1"/>
     </row>
-    <row r="53" ht="33" customHeight="1">
+    <row r="53" ht="39.75" customHeight="1">
       <c r="A53" s="1"/>
-      <c r="B53" s="22"/>
-      <c r="C53" s="22"/>
-      <c r="D53" s="22"/>
-      <c r="E53" s="22"/>
-      <c r="F53" s="16">
-        <v>2</v>
+      <c r="B53" s="60"/>
+      <c r="C53" s="41"/>
+      <c r="D53" s="41"/>
+      <c r="E53" s="41"/>
+      <c r="F53" s="17">
+        <v>3</v>
       </c>
       <c r="G53" s="14" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="H53" s="14" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="I53" s="14" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="J53" s="14" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="K53" s="1"/>
       <c r="L53" s="1"/>
@@ -3604,26 +3806,26 @@
       <c r="Y53" s="1"/>
       <c r="Z53" s="1"/>
     </row>
-    <row r="54" ht="68.25" customHeight="1">
+    <row r="54" ht="44.25" customHeight="1">
       <c r="A54" s="1"/>
-      <c r="B54" s="15"/>
-      <c r="C54" s="15"/>
-      <c r="D54" s="15"/>
-      <c r="E54" s="15"/>
-      <c r="F54" s="16">
-        <v>3</v>
+      <c r="B54" s="60"/>
+      <c r="C54" s="41"/>
+      <c r="D54" s="41"/>
+      <c r="E54" s="41"/>
+      <c r="F54" s="17">
+        <v>4</v>
       </c>
       <c r="G54" s="14" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="H54" s="14" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="I54" s="14" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="J54" s="14" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="K54" s="1"/>
       <c r="L54" s="1"/>
@@ -3642,17 +3844,27 @@
       <c r="Y54" s="1"/>
       <c r="Z54" s="1"/>
     </row>
-    <row r="55" ht="14.25" customHeight="1">
+    <row r="55" ht="36" customHeight="1">
       <c r="A55" s="1"/>
-      <c r="B55" s="23"/>
-      <c r="C55" s="23"/>
-      <c r="D55" s="23"/>
-      <c r="E55" s="23"/>
-      <c r="F55" s="23"/>
-      <c r="G55" s="23"/>
-      <c r="H55" s="23"/>
-      <c r="I55" s="23"/>
-      <c r="J55" s="23"/>
+      <c r="B55" s="61"/>
+      <c r="C55" s="62"/>
+      <c r="D55" s="62"/>
+      <c r="E55" s="62"/>
+      <c r="F55" s="17">
+        <v>5</v>
+      </c>
+      <c r="G55" s="14" t="s">
+        <v>200</v>
+      </c>
+      <c r="H55" s="14" t="s">
+        <v>201</v>
+      </c>
+      <c r="I55" s="14" t="s">
+        <v>202</v>
+      </c>
+      <c r="J55" s="14" t="s">
+        <v>203</v>
+      </c>
       <c r="K55" s="1"/>
       <c r="L55" s="1"/>
       <c r="M55" s="1"/>
@@ -3670,35 +3882,17 @@
       <c r="Y55" s="1"/>
       <c r="Z55" s="1"/>
     </row>
-    <row r="56" ht="39.75" customHeight="1">
+    <row r="56" ht="14.25" customHeight="1">
       <c r="A56" s="1"/>
-      <c r="B56" s="11" t="s">
-        <v>198</v>
-      </c>
-      <c r="C56" s="12" t="s">
-        <v>199</v>
-      </c>
-      <c r="D56" s="12" t="s">
-        <v>200</v>
-      </c>
-      <c r="E56" s="12" t="s">
-        <v>201</v>
-      </c>
-      <c r="F56" s="16">
-        <v>1</v>
-      </c>
-      <c r="G56" s="14" t="s">
-        <v>202</v>
-      </c>
-      <c r="H56" s="14" t="s">
-        <v>203</v>
-      </c>
-      <c r="I56" s="14" t="s">
-        <v>204</v>
-      </c>
-      <c r="J56" s="14" t="s">
-        <v>205</v>
-      </c>
+      <c r="B56" s="58"/>
+      <c r="C56" s="54"/>
+      <c r="D56" s="54"/>
+      <c r="E56" s="54"/>
+      <c r="F56" s="54"/>
+      <c r="G56" s="54"/>
+      <c r="H56" s="54"/>
+      <c r="I56" s="54"/>
+      <c r="J56" s="54"/>
       <c r="K56" s="1"/>
       <c r="L56" s="1"/>
       <c r="M56" s="1"/>
@@ -3716,26 +3910,34 @@
       <c r="Y56" s="1"/>
       <c r="Z56" s="1"/>
     </row>
-    <row r="57" ht="44.25" customHeight="1">
+    <row r="57" ht="47.25" customHeight="1">
       <c r="A57" s="1"/>
-      <c r="B57" s="22"/>
-      <c r="C57" s="22"/>
-      <c r="D57" s="22"/>
-      <c r="E57" s="22"/>
-      <c r="F57" s="16">
-        <v>2</v>
+      <c r="B57" s="55" t="s">
+        <v>204</v>
+      </c>
+      <c r="C57" s="12" t="s">
+        <v>205</v>
+      </c>
+      <c r="D57" s="12" t="s">
+        <v>206</v>
+      </c>
+      <c r="E57" s="12" t="s">
+        <v>207</v>
+      </c>
+      <c r="F57" s="17">
+        <v>1</v>
       </c>
       <c r="G57" s="14" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="H57" s="14" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="I57" s="14" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="J57" s="14" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="K57" s="1"/>
       <c r="L57" s="1"/>
@@ -3754,26 +3956,26 @@
       <c r="Y57" s="1"/>
       <c r="Z57" s="1"/>
     </row>
-    <row r="58" ht="36" customHeight="1">
+    <row r="58" ht="53.25" customHeight="1">
       <c r="A58" s="1"/>
-      <c r="B58" s="15"/>
-      <c r="C58" s="15"/>
-      <c r="D58" s="15"/>
-      <c r="E58" s="15"/>
-      <c r="F58" s="16">
-        <v>3</v>
+      <c r="B58" s="56"/>
+      <c r="C58" s="28"/>
+      <c r="D58" s="28"/>
+      <c r="E58" s="28"/>
+      <c r="F58" s="17">
+        <v>2</v>
       </c>
       <c r="G58" s="14" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="H58" s="14" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="I58" s="14" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="J58" s="14" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="K58" s="1"/>
       <c r="L58" s="1"/>
@@ -3792,17 +3994,27 @@
       <c r="Y58" s="1"/>
       <c r="Z58" s="1"/>
     </row>
-    <row r="59" ht="14.25" customHeight="1">
+    <row r="59" ht="53.25" customHeight="1">
       <c r="A59" s="1"/>
-      <c r="B59" s="23"/>
-      <c r="C59" s="23"/>
-      <c r="D59" s="23"/>
-      <c r="E59" s="23"/>
-      <c r="F59" s="23"/>
-      <c r="G59" s="23"/>
-      <c r="H59" s="23"/>
-      <c r="I59" s="23"/>
-      <c r="J59" s="23"/>
+      <c r="B59" s="57"/>
+      <c r="C59" s="16"/>
+      <c r="D59" s="16"/>
+      <c r="E59" s="16"/>
+      <c r="F59" s="17">
+        <v>3</v>
+      </c>
+      <c r="G59" s="14" t="s">
+        <v>216</v>
+      </c>
+      <c r="H59" s="14" t="s">
+        <v>217</v>
+      </c>
+      <c r="I59" s="14" t="s">
+        <v>218</v>
+      </c>
+      <c r="J59" s="14" t="s">
+        <v>219</v>
+      </c>
       <c r="K59" s="1"/>
       <c r="L59" s="1"/>
       <c r="M59" s="1"/>
@@ -3820,35 +4032,17 @@
       <c r="Y59" s="1"/>
       <c r="Z59" s="1"/>
     </row>
-    <row r="60" ht="47.25" customHeight="1">
+    <row r="60" ht="14.25" customHeight="1">
       <c r="A60" s="1"/>
-      <c r="B60" s="11" t="s">
-        <v>214</v>
-      </c>
-      <c r="C60" s="12" t="s">
-        <v>215</v>
-      </c>
-      <c r="D60" s="12" t="s">
-        <v>216</v>
-      </c>
-      <c r="E60" s="12" t="s">
-        <v>217</v>
-      </c>
-      <c r="F60" s="16">
-        <v>1</v>
-      </c>
-      <c r="G60" s="14" t="s">
-        <v>218</v>
-      </c>
-      <c r="H60" s="14" t="s">
-        <v>219</v>
-      </c>
-      <c r="I60" s="14" t="s">
-        <v>220</v>
-      </c>
-      <c r="J60" s="14" t="s">
-        <v>221</v>
-      </c>
+      <c r="B60" s="58"/>
+      <c r="C60" s="54"/>
+      <c r="D60" s="54"/>
+      <c r="E60" s="54"/>
+      <c r="F60" s="54"/>
+      <c r="G60" s="54"/>
+      <c r="H60" s="54"/>
+      <c r="I60" s="54"/>
+      <c r="J60" s="54"/>
       <c r="K60" s="1"/>
       <c r="L60" s="1"/>
       <c r="M60" s="1"/>
@@ -3866,26 +4060,34 @@
       <c r="Y60" s="1"/>
       <c r="Z60" s="1"/>
     </row>
-    <row r="61" ht="53.25" customHeight="1">
+    <row r="61" ht="56.25" customHeight="1">
       <c r="A61" s="1"/>
-      <c r="B61" s="22"/>
-      <c r="C61" s="22"/>
-      <c r="D61" s="22"/>
-      <c r="E61" s="22"/>
-      <c r="F61" s="16">
-        <v>2</v>
+      <c r="B61" s="55" t="s">
+        <v>220</v>
+      </c>
+      <c r="C61" s="12" t="s">
+        <v>221</v>
+      </c>
+      <c r="D61" s="12" t="s">
+        <v>222</v>
+      </c>
+      <c r="E61" s="12" t="s">
+        <v>223</v>
+      </c>
+      <c r="F61" s="17">
+        <v>1</v>
       </c>
       <c r="G61" s="14" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="H61" s="14" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="I61" s="14" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="J61" s="14" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="K61" s="1"/>
       <c r="L61" s="1"/>
@@ -3904,26 +4106,26 @@
       <c r="Y61" s="1"/>
       <c r="Z61" s="1"/>
     </row>
-    <row r="62" ht="53.25" customHeight="1">
+    <row r="62" ht="42.75">
       <c r="A62" s="1"/>
-      <c r="B62" s="15"/>
-      <c r="C62" s="15"/>
-      <c r="D62" s="15"/>
-      <c r="E62" s="15"/>
-      <c r="F62" s="16">
-        <v>3</v>
+      <c r="B62" s="56"/>
+      <c r="C62" s="28"/>
+      <c r="D62" s="28"/>
+      <c r="E62" s="28"/>
+      <c r="F62" s="17">
+        <v>2</v>
       </c>
       <c r="G62" s="14" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="H62" s="14" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="I62" s="14" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="J62" s="14" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="K62" s="1"/>
       <c r="L62" s="1"/>
@@ -3942,17 +4144,27 @@
       <c r="Y62" s="1"/>
       <c r="Z62" s="1"/>
     </row>
-    <row r="63" ht="14.25" customHeight="1">
+    <row r="63" ht="50.25" customHeight="1">
       <c r="A63" s="1"/>
-      <c r="B63" s="23"/>
-      <c r="C63" s="23"/>
-      <c r="D63" s="23"/>
-      <c r="E63" s="23"/>
-      <c r="F63" s="23"/>
-      <c r="G63" s="23"/>
-      <c r="H63" s="23"/>
-      <c r="I63" s="23"/>
-      <c r="J63" s="23"/>
+      <c r="B63" s="57"/>
+      <c r="C63" s="16"/>
+      <c r="D63" s="16"/>
+      <c r="E63" s="16"/>
+      <c r="F63" s="17">
+        <v>3</v>
+      </c>
+      <c r="G63" s="14" t="s">
+        <v>232</v>
+      </c>
+      <c r="H63" s="14" t="s">
+        <v>233</v>
+      </c>
+      <c r="I63" s="14" t="s">
+        <v>234</v>
+      </c>
+      <c r="J63" s="14" t="s">
+        <v>235</v>
+      </c>
       <c r="K63" s="1"/>
       <c r="L63" s="1"/>
       <c r="M63" s="1"/>
@@ -3970,35 +4182,17 @@
       <c r="Y63" s="1"/>
       <c r="Z63" s="1"/>
     </row>
-    <row r="64" ht="56.25" customHeight="1">
+    <row r="64" ht="18" customHeight="1">
       <c r="A64" s="1"/>
-      <c r="B64" s="11" t="s">
-        <v>230</v>
-      </c>
-      <c r="C64" s="12" t="s">
-        <v>231</v>
-      </c>
-      <c r="D64" s="12" t="s">
-        <v>232</v>
-      </c>
-      <c r="E64" s="12" t="s">
-        <v>233</v>
-      </c>
-      <c r="F64" s="16">
-        <v>1</v>
-      </c>
-      <c r="G64" s="14" t="s">
-        <v>234</v>
-      </c>
-      <c r="H64" s="14" t="s">
-        <v>235</v>
-      </c>
-      <c r="I64" s="14" t="s">
-        <v>236</v>
-      </c>
-      <c r="J64" s="14" t="s">
-        <v>237</v>
-      </c>
+      <c r="B64" s="56"/>
+      <c r="C64" s="63"/>
+      <c r="D64" s="63"/>
+      <c r="E64" s="63"/>
+      <c r="F64" s="64"/>
+      <c r="G64" s="65"/>
+      <c r="H64" s="65"/>
+      <c r="I64" s="65"/>
+      <c r="J64" s="65"/>
       <c r="K64" s="1"/>
       <c r="L64" s="1"/>
       <c r="M64" s="1"/>
@@ -4018,24 +4212,32 @@
     </row>
     <row r="65" ht="15">
       <c r="A65" s="1"/>
-      <c r="B65" s="22"/>
-      <c r="C65" s="22"/>
-      <c r="D65" s="22"/>
-      <c r="E65" s="22"/>
-      <c r="F65" s="16">
-        <v>2</v>
+      <c r="B65" s="55" t="s">
+        <v>236</v>
+      </c>
+      <c r="C65" s="12" t="s">
+        <v>237</v>
+      </c>
+      <c r="D65" s="12" t="s">
+        <v>238</v>
+      </c>
+      <c r="E65" s="12" t="s">
+        <v>239</v>
+      </c>
+      <c r="F65" s="17">
+        <v>1</v>
       </c>
       <c r="G65" s="14" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="H65" s="14" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="I65" s="14" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="J65" s="14" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="K65" s="1"/>
       <c r="L65" s="1"/>
@@ -4054,26 +4256,26 @@
       <c r="Y65" s="1"/>
       <c r="Z65" s="1"/>
     </row>
-    <row r="66" ht="50.25" customHeight="1">
+    <row r="66" ht="15">
       <c r="A66" s="1"/>
-      <c r="B66" s="15"/>
-      <c r="C66" s="15"/>
-      <c r="D66" s="15"/>
-      <c r="E66" s="15"/>
-      <c r="F66" s="16">
-        <v>3</v>
+      <c r="B66" s="56"/>
+      <c r="C66" s="28"/>
+      <c r="D66" s="28"/>
+      <c r="E66" s="28"/>
+      <c r="F66" s="17">
+        <v>2</v>
       </c>
       <c r="G66" s="14" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="H66" s="14" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="I66" s="14" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="J66" s="14" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="K66" s="1"/>
       <c r="L66" s="1"/>
@@ -4094,32 +4296,24 @@
     </row>
     <row r="67" ht="15">
       <c r="A67" s="1"/>
-      <c r="B67" s="11" t="s">
-        <v>246</v>
+      <c r="B67" s="57"/>
+      <c r="C67" s="16"/>
+      <c r="D67" s="16"/>
+      <c r="E67" s="16"/>
+      <c r="F67" s="17">
+        <v>3</v>
       </c>
-      <c r="C67" s="12" t="s">
-        <v>247</v>
-      </c>
-      <c r="D67" s="12" t="s">
+      <c r="G67" s="14" t="s">
         <v>248</v>
       </c>
-      <c r="E67" s="12" t="s">
+      <c r="H67" s="14" t="s">
         <v>249</v>
       </c>
-      <c r="F67" s="16">
-        <v>1</v>
-      </c>
-      <c r="G67" s="14" t="s">
+      <c r="I67" s="14" t="s">
         <v>250</v>
       </c>
-      <c r="H67" s="14" t="s">
+      <c r="J67" s="14" t="s">
         <v>251</v>
-      </c>
-      <c r="I67" s="14" t="s">
-        <v>252</v>
-      </c>
-      <c r="J67" s="14" t="s">
-        <v>253</v>
       </c>
       <c r="K67" s="1"/>
       <c r="L67" s="1"/>
@@ -4138,64 +4332,62 @@
       <c r="Y67" s="1"/>
       <c r="Z67" s="1"/>
     </row>
-    <row r="68" ht="15">
-      <c r="A68" s="1"/>
-      <c r="B68" s="22"/>
-      <c r="C68" s="22"/>
-      <c r="D68" s="22"/>
-      <c r="E68" s="22"/>
-      <c r="F68" s="16">
-        <v>2</v>
+    <row r="68" s="66" customFormat="1" ht="15">
+      <c r="A68" s="67"/>
+      <c r="B68" s="56"/>
+      <c r="C68" s="68"/>
+      <c r="D68" s="68"/>
+      <c r="E68" s="68"/>
+      <c r="F68" s="69"/>
+      <c r="G68" s="70"/>
+      <c r="H68" s="70"/>
+      <c r="I68" s="70"/>
+      <c r="J68" s="70"/>
+      <c r="K68" s="67"/>
+      <c r="L68" s="67"/>
+      <c r="M68" s="67"/>
+      <c r="N68" s="67"/>
+      <c r="O68" s="67"/>
+      <c r="P68" s="67"/>
+      <c r="Q68" s="67"/>
+      <c r="R68" s="67"/>
+      <c r="S68" s="67"/>
+      <c r="T68" s="67"/>
+      <c r="U68" s="67"/>
+      <c r="V68" s="67"/>
+      <c r="W68" s="67"/>
+      <c r="X68" s="67"/>
+      <c r="Y68" s="67"/>
+      <c r="Z68" s="67"/>
+    </row>
+    <row r="69" ht="15">
+      <c r="A69" s="1"/>
+      <c r="B69" s="59" t="s">
+        <v>252</v>
       </c>
-      <c r="G68" s="14" t="s">
+      <c r="C69" s="34" t="s">
+        <v>13</v>
+      </c>
+      <c r="D69" s="34" t="s">
+        <v>253</v>
+      </c>
+      <c r="E69" s="34" t="s">
         <v>254</v>
       </c>
-      <c r="H68" s="14" t="s">
+      <c r="F69" s="17">
+        <v>1</v>
+      </c>
+      <c r="G69" s="14" t="s">
         <v>255</v>
       </c>
-      <c r="I68" s="14" t="s">
+      <c r="H69" s="14" t="s">
         <v>256</v>
       </c>
-      <c r="J68" s="14" t="s">
+      <c r="I69" s="14" t="s">
         <v>257</v>
       </c>
-      <c r="K68" s="1"/>
-      <c r="L68" s="1"/>
-      <c r="M68" s="1"/>
-      <c r="N68" s="1"/>
-      <c r="O68" s="1"/>
-      <c r="P68" s="1"/>
-      <c r="Q68" s="1"/>
-      <c r="R68" s="1"/>
-      <c r="S68" s="1"/>
-      <c r="T68" s="1"/>
-      <c r="U68" s="1"/>
-      <c r="V68" s="1"/>
-      <c r="W68" s="1"/>
-      <c r="X68" s="1"/>
-      <c r="Y68" s="1"/>
-      <c r="Z68" s="1"/>
-    </row>
-    <row r="69" ht="15">
-      <c r="A69" s="1"/>
-      <c r="B69" s="15"/>
-      <c r="C69" s="15"/>
-      <c r="D69" s="15"/>
-      <c r="E69" s="15"/>
-      <c r="F69" s="16">
-        <v>3</v>
-      </c>
-      <c r="G69" s="14" t="s">
+      <c r="J69" s="14" t="s">
         <v>258</v>
-      </c>
-      <c r="H69" s="14" t="s">
-        <v>259</v>
-      </c>
-      <c r="I69" s="14" t="s">
-        <v>260</v>
-      </c>
-      <c r="J69" s="14" t="s">
-        <v>261</v>
       </c>
       <c r="K69" s="1"/>
       <c r="L69" s="1"/>
@@ -4214,17 +4406,27 @@
       <c r="Y69" s="1"/>
       <c r="Z69" s="1"/>
     </row>
-    <row r="70" ht="14.25" customHeight="1">
+    <row r="70" ht="15">
       <c r="A70" s="1"/>
-      <c r="B70" s="6"/>
-      <c r="C70" s="3"/>
-      <c r="D70" s="4"/>
-      <c r="E70" s="3"/>
-      <c r="F70" s="3"/>
-      <c r="G70" s="4"/>
-      <c r="H70" s="4"/>
-      <c r="I70" s="4"/>
-      <c r="J70" s="4"/>
+      <c r="B70" s="60"/>
+      <c r="C70" s="41"/>
+      <c r="D70" s="41"/>
+      <c r="E70" s="41"/>
+      <c r="F70" s="17">
+        <v>2</v>
+      </c>
+      <c r="G70" s="14" t="s">
+        <v>259</v>
+      </c>
+      <c r="H70" s="14" t="s">
+        <v>260</v>
+      </c>
+      <c r="I70" s="14" t="s">
+        <v>261</v>
+      </c>
+      <c r="J70" s="14" t="s">
+        <v>262</v>
+      </c>
       <c r="K70" s="1"/>
       <c r="L70" s="1"/>
       <c r="M70" s="1"/>
@@ -4242,17 +4444,27 @@
       <c r="Y70" s="1"/>
       <c r="Z70" s="1"/>
     </row>
-    <row r="71" ht="14.25" customHeight="1">
+    <row r="71" ht="15">
       <c r="A71" s="1"/>
-      <c r="B71" s="6"/>
-      <c r="C71" s="3"/>
-      <c r="D71" s="4"/>
-      <c r="E71" s="3"/>
-      <c r="F71" s="3"/>
-      <c r="G71" s="4"/>
-      <c r="H71" s="4"/>
-      <c r="I71" s="4"/>
-      <c r="J71" s="4"/>
+      <c r="B71" s="60"/>
+      <c r="C71" s="41"/>
+      <c r="D71" s="41"/>
+      <c r="E71" s="41"/>
+      <c r="F71" s="17">
+        <v>3</v>
+      </c>
+      <c r="G71" s="14" t="s">
+        <v>263</v>
+      </c>
+      <c r="H71" s="14" t="s">
+        <v>264</v>
+      </c>
+      <c r="I71" s="14" t="s">
+        <v>265</v>
+      </c>
+      <c r="J71" s="14" t="s">
+        <v>266</v>
+      </c>
       <c r="K71" s="1"/>
       <c r="L71" s="1"/>
       <c r="M71" s="1"/>
@@ -4270,17 +4482,27 @@
       <c r="Y71" s="1"/>
       <c r="Z71" s="1"/>
     </row>
-    <row r="72" ht="14.25" customHeight="1">
+    <row r="72" ht="15">
       <c r="A72" s="1"/>
-      <c r="B72" s="6"/>
-      <c r="C72" s="3"/>
-      <c r="D72" s="4"/>
-      <c r="E72" s="3"/>
-      <c r="F72" s="3"/>
-      <c r="G72" s="4"/>
-      <c r="H72" s="4"/>
-      <c r="I72" s="4"/>
-      <c r="J72" s="4"/>
+      <c r="B72" s="61"/>
+      <c r="C72" s="62"/>
+      <c r="D72" s="62"/>
+      <c r="E72" s="62"/>
+      <c r="F72" s="17">
+        <v>4</v>
+      </c>
+      <c r="G72" s="14" t="s">
+        <v>267</v>
+      </c>
+      <c r="H72" s="14" t="s">
+        <v>268</v>
+      </c>
+      <c r="I72" s="14" t="s">
+        <v>269</v>
+      </c>
+      <c r="J72" s="14" t="s">
+        <v>270</v>
+      </c>
       <c r="K72" s="1"/>
       <c r="L72" s="1"/>
       <c r="M72" s="1"/>
@@ -29862,36 +30084,8 @@
       <c r="Y985" s="1"/>
       <c r="Z985" s="1"/>
     </row>
-    <row r="986" ht="14.25" customHeight="1">
-      <c r="A986" s="1"/>
-      <c r="B986" s="6"/>
-      <c r="C986" s="3"/>
-      <c r="D986" s="4"/>
-      <c r="E986" s="3"/>
-      <c r="F986" s="3"/>
-      <c r="G986" s="4"/>
-      <c r="H986" s="4"/>
-      <c r="I986" s="4"/>
-      <c r="J986" s="4"/>
-      <c r="K986" s="1"/>
-      <c r="L986" s="1"/>
-      <c r="M986" s="1"/>
-      <c r="N986" s="1"/>
-      <c r="O986" s="1"/>
-      <c r="P986" s="1"/>
-      <c r="Q986" s="1"/>
-      <c r="R986" s="1"/>
-      <c r="S986" s="1"/>
-      <c r="T986" s="1"/>
-      <c r="U986" s="1"/>
-      <c r="V986" s="1"/>
-      <c r="W986" s="1"/>
-      <c r="X986" s="1"/>
-      <c r="Y986" s="1"/>
-      <c r="Z986" s="1"/>
-    </row>
   </sheetData>
-  <mergeCells count="83">
+  <mergeCells count="79">
     <mergeCell ref="C4:F4"/>
     <mergeCell ref="G4:J4"/>
     <mergeCell ref="B6:B7"/>
@@ -29915,66 +30109,62 @@
     <mergeCell ref="H17:H18"/>
     <mergeCell ref="I17:I18"/>
     <mergeCell ref="J17:J18"/>
-    <mergeCell ref="B20:B22"/>
-    <mergeCell ref="C20:C22"/>
-    <mergeCell ref="D20:D22"/>
-    <mergeCell ref="E20:E22"/>
-    <mergeCell ref="B24:B25"/>
-    <mergeCell ref="C24:C25"/>
-    <mergeCell ref="D24:D25"/>
-    <mergeCell ref="E24:E25"/>
-    <mergeCell ref="B27:B28"/>
-    <mergeCell ref="C27:C28"/>
-    <mergeCell ref="D27:D28"/>
-    <mergeCell ref="E27:E28"/>
-    <mergeCell ref="B30:B32"/>
-    <mergeCell ref="C30:C32"/>
-    <mergeCell ref="D30:D32"/>
-    <mergeCell ref="E30:E32"/>
-    <mergeCell ref="B34:B35"/>
-    <mergeCell ref="C34:C35"/>
-    <mergeCell ref="D34:D35"/>
-    <mergeCell ref="E34:E35"/>
-    <mergeCell ref="B37:B38"/>
-    <mergeCell ref="C37:C38"/>
-    <mergeCell ref="D37:D38"/>
-    <mergeCell ref="E37:E38"/>
-    <mergeCell ref="B40:B41"/>
-    <mergeCell ref="C40:C41"/>
-    <mergeCell ref="D40:D41"/>
-    <mergeCell ref="E40:E41"/>
-    <mergeCell ref="B43:B44"/>
-    <mergeCell ref="C43:C44"/>
-    <mergeCell ref="D43:D44"/>
-    <mergeCell ref="E43:E44"/>
-    <mergeCell ref="B46:B47"/>
-    <mergeCell ref="C46:C47"/>
-    <mergeCell ref="D46:D47"/>
-    <mergeCell ref="E46:E47"/>
-    <mergeCell ref="B49:B50"/>
-    <mergeCell ref="C49:C50"/>
-    <mergeCell ref="D49:D50"/>
-    <mergeCell ref="E49:E50"/>
-    <mergeCell ref="B52:B54"/>
-    <mergeCell ref="C52:C54"/>
-    <mergeCell ref="D52:D54"/>
-    <mergeCell ref="E52:E54"/>
-    <mergeCell ref="B56:B58"/>
-    <mergeCell ref="C56:C58"/>
-    <mergeCell ref="D56:D58"/>
-    <mergeCell ref="E56:E58"/>
-    <mergeCell ref="B60:B62"/>
-    <mergeCell ref="C60:C62"/>
-    <mergeCell ref="D60:D62"/>
-    <mergeCell ref="E60:E62"/>
-    <mergeCell ref="B64:B66"/>
-    <mergeCell ref="C64:C66"/>
-    <mergeCell ref="D64:D66"/>
-    <mergeCell ref="E64:E66"/>
-    <mergeCell ref="B67:B69"/>
-    <mergeCell ref="C67:C69"/>
-    <mergeCell ref="D67:D69"/>
-    <mergeCell ref="E67:E69"/>
+    <mergeCell ref="B22:B23"/>
+    <mergeCell ref="C22:C23"/>
+    <mergeCell ref="D22:D23"/>
+    <mergeCell ref="E22:E23"/>
+    <mergeCell ref="B25:B26"/>
+    <mergeCell ref="C25:C26"/>
+    <mergeCell ref="D25:D26"/>
+    <mergeCell ref="E25:E26"/>
+    <mergeCell ref="B28:B29"/>
+    <mergeCell ref="C28:C29"/>
+    <mergeCell ref="D28:D29"/>
+    <mergeCell ref="E28:E29"/>
+    <mergeCell ref="B31:B33"/>
+    <mergeCell ref="C31:C33"/>
+    <mergeCell ref="D31:D33"/>
+    <mergeCell ref="E31:E33"/>
+    <mergeCell ref="B35:B36"/>
+    <mergeCell ref="C35:C36"/>
+    <mergeCell ref="D35:D36"/>
+    <mergeCell ref="E35:E36"/>
+    <mergeCell ref="B38:B39"/>
+    <mergeCell ref="C38:C39"/>
+    <mergeCell ref="D38:D39"/>
+    <mergeCell ref="E38:E39"/>
+    <mergeCell ref="B41:B43"/>
+    <mergeCell ref="C41:C43"/>
+    <mergeCell ref="D41:D43"/>
+    <mergeCell ref="E41:E43"/>
+    <mergeCell ref="B45:B46"/>
+    <mergeCell ref="C45:C46"/>
+    <mergeCell ref="D45:D46"/>
+    <mergeCell ref="E45:E46"/>
+    <mergeCell ref="B48:B49"/>
+    <mergeCell ref="C48:C49"/>
+    <mergeCell ref="D48:D49"/>
+    <mergeCell ref="E48:E49"/>
+    <mergeCell ref="B51:B55"/>
+    <mergeCell ref="C51:C55"/>
+    <mergeCell ref="D51:D55"/>
+    <mergeCell ref="E51:E55"/>
+    <mergeCell ref="B57:B59"/>
+    <mergeCell ref="C57:C59"/>
+    <mergeCell ref="D57:D59"/>
+    <mergeCell ref="E57:E59"/>
+    <mergeCell ref="B61:B63"/>
+    <mergeCell ref="C61:C63"/>
+    <mergeCell ref="D61:D63"/>
+    <mergeCell ref="E61:E63"/>
+    <mergeCell ref="B65:B67"/>
+    <mergeCell ref="C65:C67"/>
+    <mergeCell ref="D65:D67"/>
+    <mergeCell ref="E65:E67"/>
+    <mergeCell ref="B69:B72"/>
+    <mergeCell ref="C69:C72"/>
+    <mergeCell ref="D69:D72"/>
+    <mergeCell ref="E69:E72"/>
   </mergeCells>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0" footer="0"/>
@@ -30000,8 +30190,8 @@
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
       <c r="A1" s="1"/>
-      <c r="B1" s="34" t="s">
-        <v>262</v>
+      <c r="B1" s="71" t="s">
+        <v>271</v>
       </c>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -30030,7 +30220,7 @@
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="1"/>
-      <c r="B2" s="35"/>
+      <c r="B2" s="72"/>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
@@ -30086,11 +30276,11 @@
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="1"/>
-      <c r="B4" s="36" t="s">
-        <v>263</v>
+      <c r="B4" s="73" t="s">
+        <v>272</v>
       </c>
-      <c r="C4" s="36" t="s">
-        <v>264</v>
+      <c r="C4" s="73" t="s">
+        <v>273</v>
       </c>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
@@ -30118,11 +30308,11 @@
     </row>
     <row r="5" ht="14.25" customHeight="1">
       <c r="A5" s="1"/>
-      <c r="B5" s="37" t="s">
+      <c r="B5" s="74" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="37" t="s">
-        <v>265</v>
+      <c r="C5" s="74" t="s">
+        <v>274</v>
       </c>
       <c r="D5" s="1"/>
       <c r="E5" s="1"/>
@@ -30150,11 +30340,11 @@
     </row>
     <row r="6" ht="14.25" customHeight="1">
       <c r="A6" s="1"/>
-      <c r="B6" s="37" t="s">
+      <c r="B6" s="74" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="37" t="s">
-        <v>266</v>
+      <c r="C6" s="74" t="s">
+        <v>275</v>
       </c>
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
@@ -30182,11 +30372,11 @@
     </row>
     <row r="7" ht="14.25" customHeight="1">
       <c r="A7" s="1"/>
-      <c r="B7" s="37" t="s">
+      <c r="B7" s="74" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="38" t="s">
-        <v>267</v>
+      <c r="C7" s="75" t="s">
+        <v>276</v>
       </c>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
@@ -30214,11 +30404,11 @@
     </row>
     <row r="8" ht="14.25" customHeight="1">
       <c r="A8" s="1"/>
-      <c r="B8" s="37" t="s">
+      <c r="B8" s="74" t="s">
         <v>6</v>
       </c>
-      <c r="C8" s="37" t="s">
-        <v>268</v>
+      <c r="C8" s="74" t="s">
+        <v>277</v>
       </c>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
@@ -30246,11 +30436,11 @@
     </row>
     <row r="9" ht="14.25" customHeight="1">
       <c r="A9" s="1"/>
-      <c r="B9" s="37" t="s">
+      <c r="B9" s="74" t="s">
         <v>7</v>
       </c>
-      <c r="C9" s="37" t="s">
-        <v>269</v>
+      <c r="C9" s="74" t="s">
+        <v>278</v>
       </c>
       <c r="D9" s="1"/>
       <c r="E9" s="1"/>
@@ -30278,11 +30468,11 @@
     </row>
     <row r="10" ht="14.25" customHeight="1">
       <c r="A10" s="1"/>
-      <c r="B10" s="37" t="s">
-        <v>270</v>
+      <c r="B10" s="74" t="s">
+        <v>279</v>
       </c>
-      <c r="C10" s="37" t="s">
-        <v>271</v>
+      <c r="C10" s="74" t="s">
+        <v>280</v>
       </c>
       <c r="D10" s="1"/>
       <c r="E10" s="1"/>
@@ -30310,11 +30500,11 @@
     </row>
     <row r="11" ht="14.25" customHeight="1">
       <c r="A11" s="1"/>
-      <c r="B11" s="37" t="s">
+      <c r="B11" s="74" t="s">
         <v>9</v>
       </c>
-      <c r="C11" s="37" t="s">
-        <v>272</v>
+      <c r="C11" s="74" t="s">
+        <v>281</v>
       </c>
       <c r="D11" s="1"/>
       <c r="E11" s="1"/>
@@ -30342,11 +30532,11 @@
     </row>
     <row r="12" ht="14.25" customHeight="1">
       <c r="A12" s="1"/>
-      <c r="B12" s="37" t="s">
+      <c r="B12" s="74" t="s">
         <v>10</v>
       </c>
-      <c r="C12" s="37" t="s">
-        <v>273</v>
+      <c r="C12" s="74" t="s">
+        <v>282</v>
       </c>
       <c r="D12" s="1"/>
       <c r="E12" s="1"/>
@@ -30374,11 +30564,11 @@
     </row>
     <row r="13" ht="14.25" customHeight="1">
       <c r="A13" s="1"/>
-      <c r="B13" s="37" t="s">
+      <c r="B13" s="74" t="s">
         <v>11</v>
       </c>
-      <c r="C13" s="37" t="s">
-        <v>274</v>
+      <c r="C13" s="74" t="s">
+        <v>283</v>
       </c>
       <c r="D13" s="1"/>
       <c r="E13" s="1"/>

</xml_diff>